<commit_message>
Oct 9 refresh: stranded pass tries every day within reach; recap keyed by day lists with computed counts; capacity row from data
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/route-days-v2/Spine-Route-Days-Kristen.xlsx
+++ b/pm/route-days-v2/Spine-Route-Days-Kristen.xlsx
@@ -2466,13 +2466,13 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Commerce Township (4) • West Bloomfield (4)</t>
+          <t>Commerce Township (4) • West Bloomfield (3)</t>
         </is>
       </c>
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=6089%20W%20MAPLE%20RD%20STE%20200%2C%20WEST%20BLOOMFIELD%2C%20Michigan&amp;waypoints=9178%20Highland%20Rd%2C%20White%20Lake%2C%20MI%20483864619%7C8355%20Highland%20Road%2C%20White%20Lake%20Charter%20Township%2C%20MI%2048386%7C1965%20Union%20Lake%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C2600%20Union%20Lake%20Rd%20suite%20140%20Commerce%20Township%2C%20Michigan%2C%2048382%7C8800%20Commerce%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C1%20William%20Carls%20Drive%2C%20Michigan%2C%2048382%7C2300%20Haggerty%20Rd%20Ste%202150%2C%20West%20Bloomfield%2C%20MI%2048323%7C6525%20W%20MAPLE%20RD%20STE%20101E%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6530%20FARMINGTON%20RD%20STE%20LL-02%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=17070%20W%2012%20MILE%20RD%20STE%20A%2C%20SOUTHFIELD%2C%20Michigan%2C%20MI%2048076&amp;waypoints=9178%20Highland%20Rd%2C%20White%20Lake%2C%20MI%20483864619%7C8355%20Highland%20Road%2C%20White%20Lake%20Charter%20Township%2C%20MI%2048386%7C1965%20Union%20Lake%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C2600%20Union%20Lake%20Rd%20suite%20140%20Commerce%20Township%2C%20Michigan%2C%2048382%7C8800%20Commerce%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C1%20William%20Carls%20Drive%2C%20Michigan%2C%2048382%7C2300%20Haggerty%20Rd%20Ste%202150%2C%20West%20Bloomfield%2C%20MI%2048323%7C6525%20W%20MAPLE%20RD%20STE%20101E%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6530%20FARMINGTON%20RD%20STE%20LL-02%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322</t>
         </is>
       </c>
     </row>
@@ -2595,13 +2595,13 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Northville (2) • Livonia (2)</t>
+          <t>Northville (2) • South Lyon (1)</t>
         </is>
       </c>
       <c r="J47" s="3" t="n"/>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2900%20Packard%20Street%2C%20Ypsilanti%2C%20Michigan%2C%2048197&amp;waypoints=23200%20Pontiac%20Trail%2C%20South%20Lyon%2C%20MI%2048178%7C422%20N%20Center%20St%2C%20Northville%2C%20Michigan%2C%2048167%7C308%20S%20Main%20St%2C%20Northville%2C%20Michigan%2C%2048167%7C38215%20W%2010%20MILE%20RD%20STE%208%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C19000%20St%20Joe%27s%20Pkwy%20suite%20200%2C%20Livonia%2C%20Michigan%2C%2048152%7C38253%20Ann%20Arbor%20Road%2C%20Livonia%2C%20Michigan%2C%2048150%7C30900%20FORD%20RD%20STE%20B%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C6149%20Elmwood%20Street%2C%20Westland%2C%20Michigan%2C%2048185%7C5624%20Research%20Drive%2C%20Canton%2C%20Michigan%2C%2048188</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2900%20Packard%20Street%2C%20Ypsilanti%2C%20Michigan%2C%2048197&amp;waypoints=23200%20Pontiac%20Trail%2C%20South%20Lyon%2C%20MI%2048178%7C422%20N%20Center%20St%2C%20Northville%2C%20Michigan%2C%2048167%7C308%20S%20Main%20St%2C%20Northville%2C%20Michigan%2C%2048167%7C38215%20W%2010%20MILE%20RD%20STE%208%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C23330%20%20Rd%20Farmington%2C%20Farmington%2C%20Michigan%2C%2048336%7C30900%20FORD%20RD%20STE%20B%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C6149%20Elmwood%20Street%2C%20Westland%2C%20Michigan%2C%2048185%7C38253%20Ann%20Arbor%20Road%2C%20Livonia%2C%20Michigan%2C%2048150%7C5624%20Research%20Drive%2C%20Canton%2C%20Michigan%2C%2048188</t>
         </is>
       </c>
     </row>
@@ -2814,13 +2814,13 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Livonia (6) • Farmington (1)</t>
+          <t>Livonia (7) • Redford (1)</t>
         </is>
       </c>
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=17070%20W%2012%20MILE%20RD%20STE%20A%2C%20SOUTHFIELD%2C%20Michigan%2C%20MI%2048076&amp;waypoints=37508%20W%20SEVEN%20MILE%20RD%2C%20LIVONIA%2C%20Michigan%7C17800%20Newburgh%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C33523%20Eight%20Mile%20Rd%20m2%2C%20Livonia%2C%20Michigan%2C%2048152%7C23330%20%20Rd%20Farmington%2C%20Farmington%2C%20Michigan%2C%2048336%7C20216%20Farmington%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C33215%20W%20Seven%20Mile%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C15604%20FARMINGTON%20RD%2C%20LIVONIA%2C%20MI%2C%2048154%7C24224%20JOY%20RD%20STE%20100%2C%20REDFORD%2C%20Michigan%7C15540%20Beech%20Daly%2C%20Redford%20Charter%20Township%2C%20Michigan%2C%2048239</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=31500%20TELEGRAPH%20RD%20STE%20115%2C%20BINGHAM%20FARMS%2C%20MI%2C%2048025&amp;waypoints=19000%20St%20Joe%27s%20Pkwy%20suite%20200%2C%20Livonia%2C%20Michigan%2C%2048152%7C17800%20Newburgh%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C37508%20W%20SEVEN%20MILE%20RD%2C%20LIVONIA%2C%20Michigan%7C33523%20Eight%20Mile%20Rd%20m2%2C%20Livonia%2C%20Michigan%2C%2048152%7C20216%20Farmington%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C33215%20W%20Seven%20Mile%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C15604%20FARMINGTON%20RD%2C%20LIVONIA%2C%20MI%2C%2048154%7C24224%20JOY%20RD%20STE%20100%2C%20REDFORD%2C%20Michigan%7C15540%20Beech%20Daly%2C%20Redford%20Charter%20Township%2C%20Michigan%2C%2048239</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2934,7 @@
         <v>10</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>5</v>
@@ -2943,17 +2943,17 @@
         <v>3</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Shelby Township (3) • Clinton Township (3)</t>
+          <t>Clinton Township (3) • Shelby Township (3)</t>
         </is>
       </c>
       <c r="J55" s="3" t="n"/>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=36750%2026%20Mile%20Rd%2C%20ste%20140%2C%20New%20Baltimore%2C%20Michigan%2C%2048047&amp;waypoints=79720%20Kidder%20Rd%20Bruce%20Township%2C%20Michigan%2C%2048065%7C57850%20Van%20Dyke%20Ave%20ste%20600%2C%20Washington%2C%20Michigan%2C%2048094%7C50720%20Schoenherr%20Rd%2C%20Shelby%20Township%2C%20MI%2048315%7C15125%2022%20Mile%20Rd%2C%20Shelby%20Township%2C%20MI%2048315%7C45640%20Schoenherr%20Rd%2C%20Shelby%20Township%2C%20Michigan%2C%2048315%7C41060%20Hayes%20Road%2C%20Clinton%20Township%2C%20Michigan%2C%2048038%7C15520%2019%20Mile%20Road%2C%20Suite%20480%2C%20Clinton%20Township%2C%20MI%2C%2048038%7C43555%20Dalcoma%20Dr%20suite%204%20Clinton%20Twp%2C%20Clinton%20Township%2C%20Michigan%2C%2048038%7C36267%2026%20Mile%20Road%2C%20Suite%203%2C%20Lenox%2C%20MI%2C%2048048</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=36750%2026%20Mile%20Rd%2C%20ste%20140%2C%20New%20Baltimore%2C%20Michigan%2C%2048047&amp;waypoints=57850%20Van%20Dyke%20Ave%20ste%20600%2C%20Washington%2C%20Michigan%2C%2048094%7C115%20E%20Long%20Lake%20Rd%2C%20Troy%2C%20MI%2048085%7C41060%20Hayes%20Road%2C%20Clinton%20Township%2C%20Michigan%2C%2048038%7C15520%2019%20Mile%20Road%2C%20Suite%20480%2C%20Clinton%20Township%2C%20MI%2C%2048038%7C43555%20Dalcoma%20Dr%20suite%204%20Clinton%20Twp%2C%20Clinton%20Township%2C%20Michigan%2C%2048038%7C45640%20Schoenherr%20Rd%2C%20Shelby%20Township%2C%20Michigan%2C%2048315%7C50720%20Schoenherr%20Rd%2C%20Shelby%20Township%2C%20MI%2048315%7C15125%2022%20Mile%20Rd%2C%20Shelby%20Township%2C%20MI%2048315%7C36267%2026%20Mile%20Road%2C%20Suite%203%2C%20Lenox%2C%20MI%2C%2048048</t>
         </is>
       </c>
     </row>
@@ -2990,13 +2990,13 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Southfield (3) • Farmington Hills (2)</t>
+          <t>Southfield (3) • West Bloomfield (2)</t>
         </is>
       </c>
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2940%20Crooks%20Rd%2C%20Rochester%20Hills%2C%20Michigan%2C%2048309&amp;waypoints=5799%20W%20MAPLE%20RD%20STE%20163%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C30055%20Northwestern%20Hwy%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C31390%20Northwestern%20Hwy.%2C%20Ste%20C%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C29355%20Northwestern%20Hwy%20%23210%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20Northwestern%20Hwy%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20NORTHWESTERN%20HWY%20STE%20120%2C%20SOUTHFIELD%2C%20MI%2C%2048034%7C31500%20TELEGRAPH%20RD%20STE%20115%2C%20BINGHAM%20FARMS%2C%20MI%2C%2048025%7C3270%20Greenfield%20Rd%2C%20Berkley%2C%20Michigan%2C%2048072%7C43700%20WOODWARD%20AVE%20STE%20206%2C%20BLOOMFIELD%2C%20Michigan%2C%20MI%2048302</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2940%20Crooks%20Rd%2C%20Rochester%20Hills%2C%20Michigan%2C%2048309&amp;waypoints=6089%20W%20MAPLE%20RD%20STE%20200%2C%20WEST%20BLOOMFIELD%2C%20Michigan%7C5799%20W%20MAPLE%20RD%20STE%20163%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C30055%20Northwestern%20Hwy%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C31390%20Northwestern%20Hwy.%2C%20Ste%20C%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C29355%20Northwestern%20Hwy%20%23210%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20Northwestern%20Hwy%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20NORTHWESTERN%20HWY%20STE%20120%2C%20SOUTHFIELD%2C%20MI%2C%2048034%7C3270%20Greenfield%20Rd%2C%20Berkley%2C%20Michigan%2C%2048072%7C43700%20WOODWARD%20AVE%20STE%20206%2C%20BLOOMFIELD%2C%20Michigan%2C%20MI%2048302</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
         <v>10</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F57" s="2" t="n">
         <v>0</v>
@@ -3029,7 +3029,7 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
@@ -3039,7 +3039,7 @@
       <c r="J57" s="3" t="n"/>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=22318%20Ford%20Road%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048127&amp;waypoints=6543%20TELEGRAPH%20RD%2C%20BLOOMFIELD%20TOWNSHIP%2C%20Michigan%7C23800%20Orchard%20Lake%20Rd%20suite%20202%2C%20Farmington%20Hills%2C%20Michigan%2C%2048336%7C23133%20Orchard%20Lake%20Rd%2C%20Farmington%2C%20Michigan%2C%2048336%7C22821%20ORCHARD%20LAKE%20RD%2C%20FARMINGTON%2C%20MI%2C%2048336%7C14700%20Farmington%20Rd%2C%20Livonia%2C%20Michigan%2C%2048154%7C36600%20Plymouth%20Road%2C%20Livonia%2C%20Michigan%2C%2048150%7C30900%20FORD%20RD%20STE%20B%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C28000%20Joy%20Road%2C%20Livonia%2C%20MI%2048150%7C27031%20W%20Warren%20St%2C%20Dearborn%20Heights%2C%20MI%2048127</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=22318%20Ford%20Road%2C%20Dearborn%20Heights%2C%20Michigan%2C%2048127&amp;waypoints=2630%20UNION%20LAKE%20RD%20STE%20100%2C%20COMMERCE%20TOWNSHIP%2C%20Michigan%7C23800%20Orchard%20Lake%20Rd%20suite%20202%2C%20Farmington%20Hills%2C%20Michigan%2C%2048336%7C23133%20Orchard%20Lake%20Rd%2C%20Farmington%2C%20Michigan%2C%2048336%7C22821%20ORCHARD%20LAKE%20RD%2C%20FARMINGTON%2C%20MI%2C%2048336%7C14700%20Farmington%20Rd%2C%20Livonia%2C%20Michigan%2C%2048154%7C36600%20Plymouth%20Road%2C%20Livonia%2C%20Michigan%2C%2048150%7C30900%20FORD%20RD%20STE%20B%2C%20GARDEN%20CITY%2C%20MI%2C%2048135%7C28000%20Joy%20Road%2C%20Livonia%2C%20MI%2048150%7C27031%20W%20Warren%20St%2C%20Dearborn%20Heights%2C%20MI%2048127</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
         <v>10</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F58" s="2" t="n">
         <v>0</v>
@@ -3072,17 +3072,17 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Commerce Township (5) • Novi (1)</t>
+          <t>Commerce Township (4) • White Lake (1)</t>
         </is>
       </c>
       <c r="J58" s="3" t="n"/>
       <c r="K58" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=2157%20ORCHARD%20LAKE%20RD%2C%20SYLVAN%20LAKE%2C%20Michigan&amp;waypoints=1%20William%20Carls%20Drive%2C%20Michigan%2C%2048382%7C26850%20PROVIDENCE%20PKWY%20STE%20455%2C%20NOVI%2C%20Michigan%7C100%20N%20POND%20DR%20STE%20C%2C%20WALLED%20LAKE%2C%20MI%2C%2048390%7C2300%20Haggerty%20Rd%20Ste%202150%2C%20West%20Bloomfield%2C%20MI%2048323%7C8800%20Commerce%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C2685%20Union%20Lake%20Rd%20Commerce%20Charter%20Twp%2C%20Commerce%20Charter%20Township%2C%20Michigan%2C%2048382%7C2630%20UNION%20LAKE%20RD%20STE%20100%2C%20COMMERCE%20TOWNSHIP%2C%20Michigan%7C2600%20Union%20Lake%20Rd%20suite%20140%20Commerce%20Township%2C%20Michigan%2C%2048382%7C1965%20Union%20Lake%20Rd%2C%20Commerce%20Township%2C%20MI%2048382</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=29877%20Telegraph%20Rd%20Ste%20200%2C%20Southfield%2C%20MI%2048034&amp;waypoints=9178%20Highland%20Rd%2C%20White%20Lake%2C%20MI%20483864619%7C1965%20Union%20Lake%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C2600%20Union%20Lake%20Rd%20suite%20140%20Commerce%20Township%2C%20Michigan%2C%2048382%7C2685%20Union%20Lake%20Rd%20Commerce%20Charter%20Twp%2C%20Commerce%20Charter%20Township%2C%20Michigan%2C%2048382%7C8800%20Commerce%20Rd%2C%20Commerce%20Township%2C%20MI%2048382%7C1%20William%20Carls%20Drive%2C%20Michigan%2C%2048382%7C26850%20PROVIDENCE%20PKWY%20STE%20455%2C%20NOVI%2C%20Michigan%7C100%20N%20POND%20DR%20STE%20C%2C%20WALLED%20LAKE%2C%20MI%2C%2048390%7C2300%20Haggerty%20Rd%20Ste%202150%2C%20West%20Bloomfield%2C%20MI%2048323</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3106,7 @@
         <v>10</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F59" s="2" t="n">
         <v>0</v>
@@ -3115,17 +3115,17 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Warren (5) • Sterling Heights (2)</t>
+          <t>Warren (6) • Southfield (2)</t>
         </is>
       </c>
       <c r="J59" s="3" t="n"/>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=22250%20PROVIDENCE%20DR%20STE%20500%2C%20SOUTHFIELD%2C%20Michigan&amp;waypoints=115%20E%20Long%20Lake%20Rd%2C%20Troy%2C%20MI%2048085%7C35200%20Dequindre%20Road%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C34764%20Dequindre%20Rd%2C%20Sterling%20Heights%2C%20MI%2048310%7C11885%20E%2012%20Mile%20Rd%20Ste%20200B%2C%20Warren%2C%20MI%2048093%7C28401%20Hoover%2C%20Warren%2C%20Michigan%2C%2048093%7C28111%20HOOVER%20RD%20STE%201A%2C%20WARREN%2C%20Michigan%7C28111%20Hoover%20Rd%2C%20Ste%205A%20Warren%2C%20Mi%2048093%2C%20Usa%2C%20Warren%2C%20MI%2048093%7C27427%20Schoenherr%20Rd%2C%20Warren%2C%20MI%2048088%7C20599%20Mack%20Ave%2C%20Grosse%20Pointe%20Woods%2C%20MI%2048236</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=27472%20Schoenherr%20Rd%20%23100%2C%20Warren%2C%20MI%2C%2048088&amp;waypoints=29829%20Telegraph%20Road%2C%20Southfield%2C%20MI%2048034%7C22250%20PROVIDENCE%20DR%20STE%20500%2C%20SOUTHFIELD%2C%20Michigan%7C34764%20Dequindre%20Rd%2C%20Sterling%20Heights%2C%20MI%2048310%7C35200%20Dequindre%20Road%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C11885%20E%2012%20Mile%20Rd%20Ste%20200B%2C%20Warren%2C%20MI%2048093%7C28401%20Hoover%2C%20Warren%2C%20Michigan%2C%2048093%7C28111%20HOOVER%20RD%20STE%201A%2C%20WARREN%2C%20Michigan%7C28111%20Hoover%20Rd%2C%20Ste%205A%20Warren%2C%20Mi%2048093%2C%20Usa%2C%20Warren%2C%20MI%2048093%7C27427%20Schoenherr%20Rd%2C%20Warren%2C%20MI%2048088</t>
         </is>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
       <c r="J60" s="3" t="n"/>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=15050%20E%20Jefferson%20Ave%20suite%20101%2C%20Grosse%20Pointe%2C%20Michigan%2C%2048230&amp;waypoints=13951%20Plumbrook%2C%20Sterling%20Heights%2C%20Michigan%2C%2048312%7C35429%20Schoenherr%20Rd%2C%20Sterling%20Heights%2C%20MI%2C%2048312%7C39200%20Garfield%20Rd%20Suite%20E%20Clinton%20Twp%2C%20Clinton%20Township%2C%20MI%2048038%7C24725%20E%20Jefferson%2C%20Saint%20Clair%20Shores%2C%20MI%2C%2048080%7C20952%20Twelve%20Mile%20Rd%20ste%20101%2C%20St.%20Clair%20Shores%2C%20Michigan%2C%2048081%7C27850%20Gratiot%20Avenue%2C%20Roseville%2C%20Michigan%2C%2048066%7C27472%20Schoenherr%20Rd%20%23100%2C%20Warren%2C%20MI%2C%2048088%7C21647%20Ryan%20Rd%2C%20Warren%2C%20MI%2C%2048091%7C19251%20Mack%20Ave%20%23333%2C%20Grosse%20Pointe%2C%20Michigan%2C%2048236</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=15050%20E%20Jefferson%20Ave%20suite%20101%2C%20Grosse%20Pointe%2C%20Michigan%2C%2048230&amp;waypoints=13951%20Plumbrook%2C%20Sterling%20Heights%2C%20Michigan%2C%2048312%7C35429%20Schoenherr%20Rd%2C%20Sterling%20Heights%2C%20MI%2C%2048312%7C39200%20Garfield%20Rd%20Suite%20E%20Clinton%20Twp%2C%20Clinton%20Township%2C%20MI%2048038%7C24725%20E%20Jefferson%2C%20Saint%20Clair%20Shores%2C%20MI%2C%2048080%7C20952%20Twelve%20Mile%20Rd%20ste%20101%2C%20St.%20Clair%20Shores%2C%20Michigan%2C%2048081%7C27850%20Gratiot%20Avenue%2C%20Roseville%2C%20Michigan%2C%2048066%7C30061%20Schoenherr%20Rd%2C%20Warren%2C%20Michigan%2C%2048088%7C21647%20Ryan%20Rd%2C%20Warren%2C%20MI%2C%2048091%7C19251%20Mack%20Ave%20%23333%2C%20Grosse%20Pointe%2C%20Michigan%2C%2048236</t>
         </is>
       </c>
     </row>
@@ -3205,13 +3205,13 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Farmington Hills (4) • West Bloomfield (3)</t>
+          <t>Farmington Hills (5) • West Bloomfield (2)</t>
         </is>
       </c>
       <c r="J61" s="3" t="n"/>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=308%20S%20Main%20St%2C%20Northville%2C%20Michigan%2C%2048167&amp;waypoints=6525%20W%20MAPLE%20RD%20STE%20101E%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6530%20FARMINGTON%20RD%20STE%20LL-02%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6089%20W%20MAPLE%20RD%20STE%20200%2C%20WEST%20BLOOMFIELD%2C%20Michigan%7C32910%20West%2013%20Mile%20Road%2C%20A101%2C%20Farmington%20Hills%2C%20MI%2048334%7C27970%20ORCHARD%20LAKE%20RD%2C%20FARMINGTON%20HILLS%2C%20Michigan%2C%2048334%7C29930%20W%2012%20MILE%20RD%20STE%206%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C29201%20Telegraph%20Rd%2C%20ste%20403%2C%20Southfield%2C%20MI%2C%2048034%7C38215%20W%2010%20MILE%20RD%20STE%208%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C422%20N%20Center%20St%2C%20Northville%2C%20Michigan%2C%2048167</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=308%20S%20Main%20St%2C%20Northville%2C%20Michigan%2C%2048167&amp;waypoints=6525%20W%20MAPLE%20RD%20STE%20101E%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6530%20FARMINGTON%20RD%20STE%20LL-02%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C32910%20West%2013%20Mile%20Road%2C%20A101%2C%20Farmington%20Hills%2C%20MI%2048334%7C27970%20ORCHARD%20LAKE%20RD%2C%20FARMINGTON%20HILLS%2C%20Michigan%2C%2048334%7C29930%20W%2012%20MILE%20RD%20STE%206%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C29201%20Telegraph%20Rd%2C%20ste%20403%2C%20Southfield%2C%20MI%2C%2048034%7C30852%20W%2010%20MILE%20RD%2C%20FARMINGTON%20HILLS%2C%20MI%2C%2048336%7C38215%20W%2010%20MILE%20RD%20STE%208%2C%20FARMINGTON%20HILLS%2C%20Michigan%7C422%20N%20Center%20St%2C%20Northville%2C%20Michigan%2C%2048167</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
       <c r="J63" s="3" t="n"/>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=26393%20Dequindre%20Rd%2C%20Madison%20Heights%2C%20Michigan%2C%2048071&amp;waypoints=44344%20Dequindre%20Rd%20Ste%20510%2C%20Sterling%20Heights%2C%20MI%20nan%7C41400%20Dequindre%20Rd%2C%20ste%20121%2C%20Sterling%20Heights%2C%20Michigan%2C%2048314%7C39333%20Van%20Dyke%20Ave%2C%20Sterling%20Heights%2C%20Mi%2048313%2C%20United%20States%2C%20Sterling%20Heights%2C%20MI%2048313%7C2567%20Metro%20Parkway%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C37450%20DeQuindre%20Rd%2C%20Sterling%20Heights%2C%20MI%2C%2048310%7C37300%20Dequindre%20Rd%20Ste%20102%2C%20Sterling%20Heights%2C%20MI%2048310%7C36040%20Dequindre%20Road%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C350%20E%2012%20Mile%20Rd%2C%20Madison%20Heights%2C%20Michigan%2C%2048071%7C28324%20Dequindre%20Road%2C%20Warren%2C%20Michigan%2C%2048092</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=39333%20Van%20Dyke%20Ave%2C%20Sterling%20Heights%2C%20Mi%2048313%2C%20United%20States%2C%20Sterling%20Heights%2C%20MI%2048313&amp;waypoints=29628%20Southfield%20Road%2C%20Southfield%2C%20Michigan%2C%2048076%7C26393%20Dequindre%20Rd%2C%20Madison%20Heights%2C%20Michigan%2C%2048071%7C350%20E%2012%20Mile%20Rd%2C%20Madison%20Heights%2C%20Michigan%2C%2048071%7C36040%20Dequindre%20Road%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C2567%20Metro%20Parkway%2C%20Sterling%20Heights%2C%20Michigan%2C%2048310%7C37300%20Dequindre%20Rd%20Ste%20102%2C%20Sterling%20Heights%2C%20MI%2048310%7C37450%20DeQuindre%20Rd%2C%20Sterling%20Heights%2C%20MI%2C%2048310%7C41400%20Dequindre%20Rd%2C%20ste%20121%2C%20Sterling%20Heights%2C%20Michigan%2C%2048314%7C44344%20Dequindre%20Rd%20Ste%20510%2C%20Sterling%20Heights%2C%20MI%20nan</t>
         </is>
       </c>
     </row>
@@ -3334,13 +3334,13 @@
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Southfield (5) • Livonia (2)</t>
+          <t>Livonia (4) • Southfield (3)</t>
         </is>
       </c>
       <c r="J64" s="3" t="n"/>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=17330%20Northland%20Park%20Ct%20Ste%20100%2C%20Southfield%2C%20MI%2048075&amp;waypoints=23330%20%20Rd%20Farmington%2C%20Farmington%2C%20Michigan%2C%2048336%7C33523%20Eight%20Mile%20Rd%20m2%2C%20Livonia%2C%20Michigan%2C%2048152%7C17940%20Farmington%20Rd%20Ste%20130%2C%20Livonia%2C%20MI%2048152%7C23700%20Orchard%20Lake%20Rd%2C%20Farmington%20Hills%2C%20MI%2C%2048336-2559%7C30852%20W%2010%20MILE%20RD%2C%20FARMINGTON%20HILLS%2C%20MI%2C%2048336%7C28670%20Telegraph%20Road%2C%20Southfield%2C%20Michigan%2C%2048034%7C29829%20Telegraph%20Road%2C%20Southfield%2C%20MI%2048034%7C29877%20Telegraph%20Rd%20Ste%20200%2C%20Southfield%2C%20MI%2048034%7C17070%20W%2012%20MILE%20RD%20STE%20A%2C%20SOUTHFIELD%2C%20Michigan%2C%20MI%2048076</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=17330%20Northland%20Park%20Ct%20Ste%20100%2C%20Southfield%2C%20MI%2048075&amp;waypoints=23330%20%20Rd%20Farmington%2C%20Farmington%2C%20Michigan%2C%2048336%7C33523%20Eight%20Mile%20Rd%20m2%2C%20Livonia%2C%20Michigan%2C%2048152%7C17940%20Farmington%20Rd%20Ste%20130%2C%20Livonia%2C%20MI%2048152%7C33215%20W%20Seven%20Mile%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C20216%20Farmington%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C23700%20Orchard%20Lake%20Rd%2C%20Farmington%20Hills%2C%20MI%2C%2048336-2559%7C28670%20Telegraph%20Road%2C%20Southfield%2C%20Michigan%2C%2048034%7C31500%20TELEGRAPH%20RD%20STE%20115%2C%20BINGHAM%20FARMS%2C%20MI%2C%2048025%7C17070%20W%2012%20MILE%20RD%20STE%20A%2C%20SOUTHFIELD%2C%20Michigan%2C%20MI%2048076</t>
         </is>
       </c>
     </row>
@@ -3377,13 +3377,13 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Livonia (3) • Farmington Hills (2)</t>
+          <t>Southfield (3) • Farmington Hills (2)</t>
         </is>
       </c>
       <c r="J65" s="3" t="n"/>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=6149%20Elmwood%20Street%2C%20Westland%2C%20Michigan%2C%2048185&amp;waypoints=9178%20Highland%20Rd%2C%20White%20Lake%2C%20MI%20483864619%7C30055%20Northwestern%20Hwy%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C31390%20Northwestern%20Hwy.%2C%20Ste%20C%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C29355%20Northwestern%20Hwy%20%23210%2C%20Southfield%2C%20Michigan%2C%2048034%7C20216%20Farmington%20Road%2C%20Livonia%2C%20Michigan%2C%2048152%7C33215%20W%20Seven%20Mile%20Rd%2C%20Livonia%2C%20Michigan%2C%2048152%7C15604%20FARMINGTON%20RD%2C%20LIVONIA%2C%20MI%2C%2048154%7C15540%20Beech%20Daly%2C%20Redford%20Charter%20Township%2C%20Michigan%2C%2048239%7C24224%20JOY%20RD%20STE%20100%2C%20REDFORD%2C%20Michigan</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=6149%20Elmwood%20Street%2C%20Westland%2C%20Michigan%2C%2048185&amp;waypoints=8355%20Highland%20Road%2C%20White%20Lake%20Charter%20Township%2C%20MI%2048386%7C30055%20Northwestern%20Hwy%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C31390%20Northwestern%20Hwy.%2C%20Ste%20C%2C%20Farmington%20Hills%2C%20Michigan%2C%2048334%7C29355%20NORTHWESTERN%20HWY%20STE%20120%2C%20SOUTHFIELD%2C%20MI%2C%2048034%7C29355%20Northwestern%20Hwy%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20Northwestern%20Hwy%20%23210%2C%20Southfield%2C%20Michigan%2C%2048034%7C15540%20Beech%20Daly%2C%20Redford%20Charter%20Township%2C%20Michigan%2C%2048239%7C24224%20JOY%20RD%20STE%20100%2C%20REDFORD%2C%20Michigan%7C15604%20FARMINGTON%20RD%2C%20LIVONIA%2C%20MI%2C%2048154</t>
         </is>
       </c>
     </row>
@@ -3592,13 +3592,13 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Warren (4) • Clinton Township (4)</t>
+          <t>Clinton Township (4) • Sterling Heights (3)</t>
         </is>
       </c>
       <c r="J70" s="3" t="n"/>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=43600%20Garfield%20Rd%2C%20Clinton%20Township%2C%20Michigan%2C%2048038&amp;waypoints=38300%20Van%20Dyke%20Ave%2C%20Ste%20105%2C%20Sterling%20Heights%2C%20MI%2048312%7C4600%2014%20Mile%20Rd%20ste%201%2C%20Warren%2C%20Michigan%2C%2048092%7C11270%20East%20Thirteen%20Mile%20Road%2C%20Warren%2C%20Michigan%2C%2048093%7C29703%20HOOVER%20RD%20STE%20A%2C%20WARREN%2C%20Michigan%2C%2048093%7C30061%20Schoenherr%20Rd%2C%20Warren%2C%20Michigan%2C%2048088%7C13951%20Plumbrook%2C%20Sterling%20Heights%2C%20Michigan%2C%2048312%7C39200%20Garfield%20Rd%20Suite%20E%20Clinton%20Twp%2C%20Clinton%20Township%2C%20MI%2048038%7C15520%2019%20Mile%20Road%2C%20Suite%20480%2C%20Clinton%20Township%2C%20MI%2C%2048038%7C15500%2019%20Mile%20Rd%20Suite%20300%2C%20Clinton%20Township%2C%20MI%2048038</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=20599%20Mack%20Ave%2C%20Grosse%20Pointe%20Woods%2C%20MI%2048236&amp;waypoints=38300%20Van%20Dyke%20Ave%2C%20Ste%20105%2C%20Sterling%20Heights%2C%20MI%2048312%7C15500%2019%20Mile%20Rd%20Suite%20300%2C%20Clinton%20Township%2C%20MI%2048038%7C15520%2019%20Mile%20Road%2C%20Suite%20480%2C%20Clinton%20Township%2C%20MI%2C%2048038%7C43600%20Garfield%20Rd%2C%20Clinton%20Township%2C%20Michigan%2C%2048038%7C39200%20Garfield%20Rd%20Suite%20E%20Clinton%20Twp%2C%20Clinton%20Township%2C%20MI%2048038%7C13951%20Plumbrook%2C%20Sterling%20Heights%2C%20Michigan%2C%2048312%7C35429%20Schoenherr%20Rd%2C%20Sterling%20Heights%2C%20MI%2C%2048312%7C11270%20East%20Thirteen%20Mile%20Road%2C%20Warren%2C%20Michigan%2C%2048093%7C29703%20HOOVER%20RD%20STE%20A%2C%20WARREN%2C%20Michigan%2C%2048093</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
         <v>10</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" s="2" t="n">
         <v>0</v>
@@ -3674,17 +3674,17 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Southfield (2) • White Lake Charter Township (1)</t>
+          <t>West Bloomfield (2) • Troy (2)</t>
         </is>
       </c>
       <c r="J72" s="3" t="n"/>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=43700%20WOODWARD%20AVE%20STE%20206%2C%20BLOOMFIELD%2C%20Michigan%2C%20MI%2048302&amp;waypoints=8355%20Highland%20Road%2C%20White%20Lake%20Charter%20Township%2C%20MI%2048386%7C5799%20W%20MAPLE%20RD%20STE%20163%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C23800%20Orchard%20Lake%20Rd%20suite%20202%2C%20Farmington%20Hills%2C%20Michigan%2C%2048336%7C29355%20Northwestern%20Hwy%2C%20Southfield%2C%20Michigan%2C%2048034%7C29355%20NORTHWESTERN%20HWY%20STE%20120%2C%20SOUTHFIELD%2C%20MI%2C%2048034%7C31500%20TELEGRAPH%20RD%20STE%20115%2C%20BINGHAM%20FARMS%2C%20MI%2C%2048025%7C3270%20Greenfield%20Rd%2C%20Berkley%2C%20Michigan%2C%2048072%7C31005%20John%20R%20Rd%20suite%20a%2C%20Madison%20Heights%2C%20Michigan%2C%2048071%7C3456%20Rochester%20Rd%2C%20Troy%2C%20Michigan%2C%2048083</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;travelmode=driving&amp;dir_action=navigate&amp;destination=23133%20Orchard%20Lake%20Rd%2C%20Farmington%2C%20Michigan%2C%2048336&amp;waypoints=6089%20W%20MAPLE%20RD%20STE%20200%2C%20WEST%20BLOOMFIELD%2C%20Michigan%7C5799%20W%20MAPLE%20RD%20STE%20163%2C%20WEST%20BLOOMFIELD%2C%20MI%2C%2048322%7C6543%20TELEGRAPH%20RD%2C%20BLOOMFIELD%20TOWNSHIP%2C%20Michigan%7C43700%20WOODWARD%20AVE%20STE%20206%2C%20BLOOMFIELD%2C%20Michigan%2C%20MI%2048302%7C115%20E%20Long%20Lake%20Rd%2C%20Troy%2C%20MI%2048085%7C3456%20Rochester%20Rd%2C%20Troy%2C%20Michigan%2C%2048083%7C31005%20John%20R%20Rd%20suite%20a%2C%20Madison%20Heights%2C%20Michigan%2C%2048071%7C3270%20Greenfield%20Rd%2C%20Berkley%2C%20Michigan%2C%2048072%7C23800%20Orchard%20Lake%20Rd%20suite%20202%2C%20Farmington%20Hills%2C%20Michigan%2C%2048336</t>
         </is>
       </c>
     </row>
@@ -27485,7 +27485,7 @@
       </c>
       <c r="D390" s="3" t="inlineStr">
         <is>
-          <t>📝 Center For Hollistic Medicine</t>
+          <t>📝 SOUTHFIELD MEDICAL CLINIC AND PREMIER URGENT CARE AND WALK IN CLINIC</t>
         </is>
       </c>
       <c r="E390" s="3" t="inlineStr">
@@ -27500,17 +27500,17 @@
       </c>
       <c r="G390" s="2" t="inlineStr">
         <is>
-          <t>42b038b0-949b-46be-8843-e02868bb894a</t>
+          <t>297a710c-01f5-41e0-9ffc-d1df69e9329d</t>
         </is>
       </c>
       <c r="H390" s="2" t="inlineStr">
         <is>
-          <t>Other / Verify</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="I390" s="2" t="inlineStr">
         <is>
-          <t>Not sure</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J390" s="2" t="n">
@@ -27518,12 +27518,12 @@
       </c>
       <c r="K390" s="2" t="inlineStr">
         <is>
-          <t>West Bloomfield</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L390" s="3" t="inlineStr">
         <is>
-          <t>6089 W MAPLE RD STE 200, WEST BLOOMFIELD, Michigan</t>
+          <t>17070 W 12 MILE RD STE A, SOUTHFIELD, Michigan, MI 48076</t>
         </is>
       </c>
       <c r="M390" s="3" t="n"/>
@@ -28985,12 +28985,12 @@
       </c>
       <c r="D415" s="3" t="inlineStr">
         <is>
-          <t>📝 Trinity IHA Primary Care - Schoolcraft Campus</t>
+          <t>📝 Ivy Rehab - Farmington</t>
         </is>
       </c>
       <c r="E415" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 11</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F415" s="2" t="inlineStr">
@@ -29000,12 +29000,12 @@
       </c>
       <c r="G415" s="2" t="inlineStr">
         <is>
-          <t>4b1cacba-85fb-4f63-8660-c3314cf72677</t>
+          <t>d1393500-eb13-4514-9e0b-427f872ffa8b</t>
         </is>
       </c>
       <c r="H415" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="I415" s="2" t="inlineStr">
@@ -29014,16 +29014,16 @@
         </is>
       </c>
       <c r="J415" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K415" s="2" t="inlineStr">
         <is>
-          <t>Livonia</t>
+          <t>Farmington</t>
         </is>
       </c>
       <c r="L415" s="3" t="inlineStr">
         <is>
-          <t>19000 St Joe's Pkwy suite 200, Livonia, Michigan, 48152</t>
+          <t>23330  Rd Farmington, Farmington, Michigan, 48336</t>
         </is>
       </c>
       <c r="M415" s="3" t="n"/>
@@ -29045,12 +29045,12 @@
       </c>
       <c r="D416" s="3" t="inlineStr">
         <is>
-          <t>📝 Park Medical Centers</t>
+          <t>📝 GARDEN CITY FAMILY PHYSICIANS</t>
         </is>
       </c>
       <c r="E416" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 27</t>
+          <t>Tier 1 producer · last check-in Sep 1</t>
         </is>
       </c>
       <c r="F416" s="2" t="inlineStr">
@@ -29060,7 +29060,7 @@
       </c>
       <c r="G416" s="2" t="inlineStr">
         <is>
-          <t>92913d4d-edc4-462b-aecf-ef3f54198f09</t>
+          <t>be4c4280-49d5-443c-b413-3471ee753d27</t>
         </is>
       </c>
       <c r="H416" s="2" t="inlineStr">
@@ -29074,16 +29074,16 @@
         </is>
       </c>
       <c r="J416" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
-          <t>Livonia</t>
+          <t>Garden City</t>
         </is>
       </c>
       <c r="L416" s="3" t="inlineStr">
         <is>
-          <t>38253 Ann Arbor Road, Livonia, Michigan, 48150</t>
+          <t>30900 FORD RD STE B, GARDEN CITY, MI, 48135</t>
         </is>
       </c>
       <c r="M416" s="3" t="n"/>
@@ -29105,7 +29105,7 @@
       </c>
       <c r="D417" s="3" t="inlineStr">
         <is>
-          <t>📝 GARDEN CITY FAMILY PHYSICIANS</t>
+          <t>📝 Greg Monroe DO PC</t>
         </is>
       </c>
       <c r="E417" s="3" t="inlineStr">
@@ -29120,7 +29120,7 @@
       </c>
       <c r="G417" s="2" t="inlineStr">
         <is>
-          <t>be4c4280-49d5-443c-b413-3471ee753d27</t>
+          <t>4de0cfd4-93f7-4efa-a4ed-25a3ceaf173b</t>
         </is>
       </c>
       <c r="H417" s="2" t="inlineStr">
@@ -29134,16 +29134,16 @@
         </is>
       </c>
       <c r="J417" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K417" s="2" t="inlineStr">
         <is>
-          <t>Garden City</t>
+          <t>Westland</t>
         </is>
       </c>
       <c r="L417" s="3" t="inlineStr">
         <is>
-          <t>30900 FORD RD STE B, GARDEN CITY, MI, 48135</t>
+          <t>6149 Elmwood Street, Westland, Michigan, 48185</t>
         </is>
       </c>
       <c r="M417" s="3" t="n"/>
@@ -29165,12 +29165,12 @@
       </c>
       <c r="D418" s="3" t="inlineStr">
         <is>
-          <t>📝 Greg Monroe DO PC</t>
+          <t>📝 Park Medical Centers</t>
         </is>
       </c>
       <c r="E418" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 1</t>
+          <t>Tier 1 producer · last check-in Aug 27</t>
         </is>
       </c>
       <c r="F418" s="2" t="inlineStr">
@@ -29180,7 +29180,7 @@
       </c>
       <c r="G418" s="2" t="inlineStr">
         <is>
-          <t>4de0cfd4-93f7-4efa-a4ed-25a3ceaf173b</t>
+          <t>92913d4d-edc4-462b-aecf-ef3f54198f09</t>
         </is>
       </c>
       <c r="H418" s="2" t="inlineStr">
@@ -29194,16 +29194,16 @@
         </is>
       </c>
       <c r="J418" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
-          <t>Westland</t>
+          <t>Livonia</t>
         </is>
       </c>
       <c r="L418" s="3" t="inlineStr">
         <is>
-          <t>6149 Elmwood Street, Westland, Michigan, 48185</t>
+          <t>38253 Ann Arbor Road, Livonia, Michigan, 48150</t>
         </is>
       </c>
       <c r="M418" s="3" t="n"/>
@@ -31445,12 +31445,12 @@
       </c>
       <c r="D456" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Health Medical Center - Seven Mile Road</t>
+          <t>📝 Trinity IHA Primary Care - Schoolcraft Campus</t>
         </is>
       </c>
       <c r="E456" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 11</t>
+          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 11</t>
         </is>
       </c>
       <c r="F456" s="2" t="inlineStr">
@@ -31460,7 +31460,7 @@
       </c>
       <c r="G456" s="2" t="inlineStr">
         <is>
-          <t>44019f00-063b-4cdc-83d9-96ee51f8c6e3</t>
+          <t>4b1cacba-85fb-4f63-8660-c3314cf72677</t>
         </is>
       </c>
       <c r="H456" s="2" t="inlineStr">
@@ -31483,7 +31483,7 @@
       </c>
       <c r="L456" s="3" t="inlineStr">
         <is>
-          <t>37508 W SEVEN MILE RD, LIVONIA, Michigan</t>
+          <t>19000 St Joe's Pkwy suite 200, Livonia, Michigan, 48152</t>
         </is>
       </c>
       <c r="M456" s="3" t="n"/>
@@ -31565,12 +31565,12 @@
       </c>
       <c r="D458" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Health - Family Medicine 8 Mile Livonia</t>
+          <t>📝 Henry Ford Health Medical Center - Seven Mile Road</t>
         </is>
       </c>
       <c r="E458" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 16</t>
+          <t>Tier 1 producer · last check-in Sep 11</t>
         </is>
       </c>
       <c r="F458" s="2" t="inlineStr">
@@ -31580,7 +31580,7 @@
       </c>
       <c r="G458" s="2" t="inlineStr">
         <is>
-          <t>22476694-35cd-4d2b-b17f-07cee1f1db4b</t>
+          <t>44019f00-063b-4cdc-83d9-96ee51f8c6e3</t>
         </is>
       </c>
       <c r="H458" s="2" t="inlineStr">
@@ -31603,7 +31603,7 @@
       </c>
       <c r="L458" s="3" t="inlineStr">
         <is>
-          <t>33523 Eight Mile Rd m2, Livonia, Michigan, 48152</t>
+          <t>37508 W SEVEN MILE RD, LIVONIA, Michigan</t>
         </is>
       </c>
       <c r="M458" s="3" t="n"/>
@@ -31625,12 +31625,12 @@
       </c>
       <c r="D459" s="3" t="inlineStr">
         <is>
-          <t>📝 Ivy Rehab - Farmington</t>
+          <t>📝 Henry Ford Health - Family Medicine 8 Mile Livonia</t>
         </is>
       </c>
       <c r="E459" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 19</t>
+          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 16</t>
         </is>
       </c>
       <c r="F459" s="2" t="inlineStr">
@@ -31640,12 +31640,12 @@
       </c>
       <c r="G459" s="2" t="inlineStr">
         <is>
-          <t>d1393500-eb13-4514-9e0b-427f872ffa8b</t>
+          <t>22476694-35cd-4d2b-b17f-07cee1f1db4b</t>
         </is>
       </c>
       <c r="H459" s="2" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I459" s="2" t="inlineStr">
@@ -31654,16 +31654,16 @@
         </is>
       </c>
       <c r="J459" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K459" s="2" t="inlineStr">
         <is>
-          <t>Farmington</t>
+          <t>Livonia</t>
         </is>
       </c>
       <c r="L459" s="3" t="inlineStr">
         <is>
-          <t>23330  Rd Farmington, Farmington, Michigan, 48336</t>
+          <t>33523 Eight Mile Rd m2, Livonia, Michigan, 48152</t>
         </is>
       </c>
       <c r="M459" s="3" t="n"/>
@@ -31985,7 +31985,7 @@
       </c>
       <c r="D465" s="3" t="inlineStr">
         <is>
-          <t>📝 SOUTHFIELD MEDICAL CLINIC AND PREMIER URGENT CARE AND WALK IN CLINIC</t>
+          <t>📝 ROSE MEDICINE</t>
         </is>
       </c>
       <c r="E465" s="3" t="inlineStr">
@@ -32000,12 +32000,12 @@
       </c>
       <c r="G465" s="2" t="inlineStr">
         <is>
-          <t>297a710c-01f5-41e0-9ffc-d1df69e9329d</t>
+          <t>9c2f2817-fae0-4fb0-b943-376aef6fc719</t>
         </is>
       </c>
       <c r="H465" s="2" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I465" s="2" t="inlineStr">
@@ -32018,12 +32018,12 @@
       </c>
       <c r="K465" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Bingham Farms</t>
         </is>
       </c>
       <c r="L465" s="3" t="inlineStr">
         <is>
-          <t>17070 W 12 MILE RD STE A, SOUTHFIELD, Michigan, MI 48076</t>
+          <t>31500 TELEGRAPH RD STE 115, BINGHAM FARMS, MI, 48025</t>
         </is>
       </c>
       <c r="M465" s="3" t="n"/>
@@ -33005,27 +33005,27 @@
       </c>
       <c r="D482" s="3" t="inlineStr">
         <is>
-          <t>Total Urgent Care - Romeo</t>
+          <t>📝 Academic Internal Medicine (Ascension)</t>
         </is>
       </c>
       <c r="E482" s="3" t="inlineStr">
         <is>
-          <t>Prospect first-touch</t>
+          <t>Tier 3 · last check-in Aug 24</t>
         </is>
       </c>
       <c r="F482" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 3</t>
         </is>
       </c>
       <c r="G482" s="2" t="inlineStr">
         <is>
-          <t>faf664cc-930b-4471-8786-7027f805cedd</t>
+          <t>97ae4125-fd10-47de-8cae-c053e42232d0</t>
         </is>
       </c>
       <c r="H482" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I482" s="2" t="inlineStr">
@@ -33038,12 +33038,12 @@
       </c>
       <c r="K482" s="2" t="inlineStr">
         <is>
-          <t>Bruce Township</t>
+          <t>Washington</t>
         </is>
       </c>
       <c r="L482" s="3" t="inlineStr">
         <is>
-          <t>79720 Kidder Rd Bruce Township, Michigan, 48065</t>
+          <t>57850 Van Dyke Ave ste 600, Washington, Michigan, 48094</t>
         </is>
       </c>
       <c r="M482" s="3" t="n"/>
@@ -33065,45 +33065,45 @@
       </c>
       <c r="D483" s="3" t="inlineStr">
         <is>
-          <t>📝 Academic Internal Medicine (Ascension)</t>
+          <t>Oakland Medical Center</t>
         </is>
       </c>
       <c r="E483" s="3" t="inlineStr">
         <is>
-          <t>Tier 3 · last check-in Aug 24</t>
+          <t>Tier 1 producer · last check-in Oct 1</t>
         </is>
       </c>
       <c r="F483" s="2" t="inlineStr">
         <is>
-          <t>Tier 3</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G483" s="2" t="inlineStr">
         <is>
-          <t>97ae4125-fd10-47de-8cae-c053e42232d0</t>
+          <t>77bba5d4-d050-4705-b292-6e3a8a78dec8</t>
         </is>
       </c>
       <c r="H483" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I483" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J483" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K483" s="2" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="L483" s="3" t="inlineStr">
         <is>
-          <t>57850 Van Dyke Ave ste 600, Washington, Michigan, 48094</t>
+          <t>115 E Long Lake Rd, Troy, MI 48085</t>
         </is>
       </c>
       <c r="M483" s="3" t="n"/>
@@ -33125,32 +33125,32 @@
       </c>
       <c r="D484" s="3" t="inlineStr">
         <is>
-          <t>Pediatric Consultants of Troy - Shelby Township</t>
+          <t>📝 Macomb Spine Care</t>
         </is>
       </c>
       <c r="E484" s="3" t="inlineStr">
         <is>
-          <t>Tier 2 ortho · tier Prospect→Tier 2 (Sep 22) · last check-in Jun 22</t>
+          <t>Tier 3 · last check-in Aug 24</t>
         </is>
       </c>
       <c r="F484" s="2" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 3</t>
         </is>
       </c>
       <c r="G484" s="2" t="inlineStr">
         <is>
-          <t>7f486a16-5999-4a69-b80d-9de7d1f85a2d</t>
+          <t>c3d66a4c-f046-43dd-ae93-ae4aabe95524</t>
         </is>
       </c>
       <c r="H484" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="I484" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J484" s="2" t="n">
@@ -33158,12 +33158,12 @@
       </c>
       <c r="K484" s="2" t="inlineStr">
         <is>
-          <t>Shelby Township</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L484" s="3" t="inlineStr">
         <is>
-          <t>50720 Schoenherr Rd, Shelby Township, MI 48315</t>
+          <t>41060 Hayes Road, Clinton Township, Michigan, 48038</t>
         </is>
       </c>
       <c r="M484" s="3" t="n"/>
@@ -33185,45 +33185,45 @@
       </c>
       <c r="D485" s="3" t="inlineStr">
         <is>
-          <t>Shelby Pediatric Associates &amp; Child Lung Center</t>
+          <t>📝 Macomb Internal Medicine</t>
         </is>
       </c>
       <c r="E485" s="3" t="inlineStr">
         <is>
-          <t>Tier 2 ortho · last check-in Jun 22</t>
+          <t>Tier 1 producer · last check-in Jul 10</t>
         </is>
       </c>
       <c r="F485" s="2" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G485" s="2" t="inlineStr">
         <is>
-          <t>cbb6770d-0a7e-4610-a0a9-34566000818b</t>
+          <t>5271bbd8-dfe5-4d54-a0a2-f5547050cafe</t>
         </is>
       </c>
       <c r="H485" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I485" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J485" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K485" s="2" t="inlineStr">
         <is>
-          <t>Shelby Township</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L485" s="3" t="inlineStr">
         <is>
-          <t>15125 22 Mile Rd, Shelby Township, MI 48315</t>
+          <t>15520 19 Mile Road, Suite 480, Clinton Township, MI, 48038</t>
         </is>
       </c>
       <c r="M485" s="3" t="n"/>
@@ -33245,7 +33245,7 @@
       </c>
       <c r="D486" s="3" t="inlineStr">
         <is>
-          <t>📝 Cornerstone St. Clair Internists</t>
+          <t>📝 David S Weingarden MD &amp; Associates</t>
         </is>
       </c>
       <c r="E486" s="3" t="inlineStr">
@@ -33260,12 +33260,12 @@
       </c>
       <c r="G486" s="2" t="inlineStr">
         <is>
-          <t>cc9cf66d-2e3c-4e56-9aeb-85ba4b7e600c</t>
+          <t>ec2dcadc-ce63-4324-aea0-52ae2b2bdd91</t>
         </is>
       </c>
       <c r="H486" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Orthopedic</t>
         </is>
       </c>
       <c r="I486" s="2" t="inlineStr">
@@ -33278,12 +33278,12 @@
       </c>
       <c r="K486" s="2" t="inlineStr">
         <is>
-          <t>Shelby Township</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L486" s="3" t="inlineStr">
         <is>
-          <t>45640 Schoenherr Rd, Shelby Township, Michigan, 48315</t>
+          <t>43555 Dalcoma Dr suite 4 Clinton Twp, Clinton Township, Michigan, 48038</t>
         </is>
       </c>
       <c r="M486" s="3" t="n"/>
@@ -33305,27 +33305,27 @@
       </c>
       <c r="D487" s="3" t="inlineStr">
         <is>
-          <t>📝 Macomb Spine Care</t>
+          <t>📝 Cornerstone St. Clair Internists</t>
         </is>
       </c>
       <c r="E487" s="3" t="inlineStr">
         <is>
-          <t>Tier 3 · last check-in Aug 24</t>
+          <t>Tier 2 ortho · last check-in Aug 24</t>
         </is>
       </c>
       <c r="F487" s="2" t="inlineStr">
         <is>
-          <t>Tier 3</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="G487" s="2" t="inlineStr">
         <is>
-          <t>c3d66a4c-f046-43dd-ae93-ae4aabe95524</t>
+          <t>cc9cf66d-2e3c-4e56-9aeb-85ba4b7e600c</t>
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I487" s="2" t="inlineStr">
@@ -33338,12 +33338,12 @@
       </c>
       <c r="K487" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Shelby Township</t>
         </is>
       </c>
       <c r="L487" s="3" t="inlineStr">
         <is>
-          <t>41060 Hayes Road, Clinton Township, Michigan, 48038</t>
+          <t>45640 Schoenherr Rd, Shelby Township, Michigan, 48315</t>
         </is>
       </c>
       <c r="M487" s="3" t="n"/>
@@ -33365,45 +33365,45 @@
       </c>
       <c r="D488" s="3" t="inlineStr">
         <is>
-          <t>📝 Macomb Internal Medicine</t>
+          <t>Pediatric Consultants of Troy - Shelby Township</t>
         </is>
       </c>
       <c r="E488" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Jul 10</t>
+          <t>Tier 2 ortho · tier Prospect→Tier 2 (Sep 22) · last check-in Jun 22</t>
         </is>
       </c>
       <c r="F488" s="2" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="G488" s="2" t="inlineStr">
         <is>
-          <t>5271bbd8-dfe5-4d54-a0a2-f5547050cafe</t>
+          <t>7f486a16-5999-4a69-b80d-9de7d1f85a2d</t>
         </is>
       </c>
       <c r="H488" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I488" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J488" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K488" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Shelby Township</t>
         </is>
       </c>
       <c r="L488" s="3" t="inlineStr">
         <is>
-          <t>15520 19 Mile Road, Suite 480, Clinton Township, MI, 48038</t>
+          <t>50720 Schoenherr Rd, Shelby Township, MI 48315</t>
         </is>
       </c>
       <c r="M488" s="3" t="n"/>
@@ -33425,12 +33425,12 @@
       </c>
       <c r="D489" s="3" t="inlineStr">
         <is>
-          <t>📝 David S Weingarden MD &amp; Associates</t>
+          <t>Shelby Pediatric Associates &amp; Child Lung Center</t>
         </is>
       </c>
       <c r="E489" s="3" t="inlineStr">
         <is>
-          <t>Tier 2 ortho · last check-in Aug 24</t>
+          <t>Tier 2 ortho · last check-in Jun 22</t>
         </is>
       </c>
       <c r="F489" s="2" t="inlineStr">
@@ -33440,17 +33440,17 @@
       </c>
       <c r="G489" s="2" t="inlineStr">
         <is>
-          <t>ec2dcadc-ce63-4324-aea0-52ae2b2bdd91</t>
+          <t>cbb6770d-0a7e-4610-a0a9-34566000818b</t>
         </is>
       </c>
       <c r="H489" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I489" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J489" s="2" t="n">
@@ -33458,12 +33458,12 @@
       </c>
       <c r="K489" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Shelby Township</t>
         </is>
       </c>
       <c r="L489" s="3" t="inlineStr">
         <is>
-          <t>43555 Dalcoma Dr suite 4 Clinton Twp, Clinton Township, Michigan, 48038</t>
+          <t>15125 22 Mile Rd, Shelby Township, MI 48315</t>
         </is>
       </c>
       <c r="M489" s="3" t="n"/>
@@ -33605,7 +33605,7 @@
       </c>
       <c r="D492" s="3" t="inlineStr">
         <is>
-          <t>📝 MARY LEE, MD, PC</t>
+          <t>📝 Center For Hollistic Medicine</t>
         </is>
       </c>
       <c r="E492" s="3" t="inlineStr">
@@ -33620,17 +33620,17 @@
       </c>
       <c r="G492" s="2" t="inlineStr">
         <is>
-          <t>d62a30ae-10fe-4408-a2cc-7b0aa9422bb8</t>
+          <t>42b038b0-949b-46be-8843-e02868bb894a</t>
         </is>
       </c>
       <c r="H492" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Other / Verify</t>
         </is>
       </c>
       <c r="I492" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not sure</t>
         </is>
       </c>
       <c r="J492" s="2" t="n">
@@ -33643,7 +33643,7 @@
       </c>
       <c r="L492" s="3" t="inlineStr">
         <is>
-          <t>5799 W MAPLE RD STE 163, WEST BLOOMFIELD, MI, 48322</t>
+          <t>6089 W MAPLE RD STE 200, WEST BLOOMFIELD, Michigan</t>
         </is>
       </c>
       <c r="M492" s="3" t="n"/>
@@ -33665,12 +33665,12 @@
       </c>
       <c r="D493" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Primary Care Center - 160</t>
+          <t>📝 MARY LEE, MD, PC</t>
         </is>
       </c>
       <c r="E493" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 23</t>
+          <t>Tier 1 producer · last check-in Sep 10</t>
         </is>
       </c>
       <c r="F493" s="2" t="inlineStr">
@@ -33680,7 +33680,7 @@
       </c>
       <c r="G493" s="2" t="inlineStr">
         <is>
-          <t>b6033c7f-ac4e-4957-b3b0-519077da6c8d</t>
+          <t>d62a30ae-10fe-4408-a2cc-7b0aa9422bb8</t>
         </is>
       </c>
       <c r="H493" s="2" t="inlineStr">
@@ -33694,16 +33694,16 @@
         </is>
       </c>
       <c r="J493" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K493" s="2" t="inlineStr">
         <is>
-          <t>Farmington Hills</t>
+          <t>West Bloomfield</t>
         </is>
       </c>
       <c r="L493" s="3" t="inlineStr">
         <is>
-          <t>30055 Northwestern Hwy, Farmington Hills, Michigan, 48334</t>
+          <t>5799 W MAPLE RD STE 163, WEST BLOOMFIELD, MI, 48322</t>
         </is>
       </c>
       <c r="M493" s="3" t="n"/>
@@ -33725,7 +33725,7 @@
       </c>
       <c r="D494" s="3" t="inlineStr">
         <is>
-          <t>📝 Levine Clinic of Chiropractic</t>
+          <t>📝 Henry Ford Primary Care Center - 160</t>
         </is>
       </c>
       <c r="E494" s="3" t="inlineStr">
@@ -33740,12 +33740,12 @@
       </c>
       <c r="G494" s="2" t="inlineStr">
         <is>
-          <t>e19f7675-d86b-445b-ad8d-c06409bfde92</t>
+          <t>b6033c7f-ac4e-4957-b3b0-519077da6c8d</t>
         </is>
       </c>
       <c r="H494" s="2" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I494" s="2" t="inlineStr">
@@ -33754,7 +33754,7 @@
         </is>
       </c>
       <c r="J494" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K494" s="2" t="inlineStr">
         <is>
@@ -33763,7 +33763,7 @@
       </c>
       <c r="L494" s="3" t="inlineStr">
         <is>
-          <t>31390 Northwestern Hwy., Ste C, Farmington Hills, Michigan, 48334</t>
+          <t>30055 Northwestern Hwy, Farmington Hills, Michigan, 48334</t>
         </is>
       </c>
       <c r="M494" s="3" t="n"/>
@@ -33785,12 +33785,12 @@
       </c>
       <c r="D495" s="3" t="inlineStr">
         <is>
-          <t>📝 Corewell Internal Medicine Southfield</t>
+          <t>📝 Levine Clinic of Chiropractic</t>
         </is>
       </c>
       <c r="E495" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 29</t>
+          <t>Tier 1 producer · last check-in Sep 23</t>
         </is>
       </c>
       <c r="F495" s="2" t="inlineStr">
@@ -33800,12 +33800,12 @@
       </c>
       <c r="G495" s="2" t="inlineStr">
         <is>
-          <t>5eb6a409-5e7b-430f-a462-af3a919cfc22</t>
+          <t>e19f7675-d86b-445b-ad8d-c06409bfde92</t>
         </is>
       </c>
       <c r="H495" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="I495" s="2" t="inlineStr">
@@ -33814,16 +33814,16 @@
         </is>
       </c>
       <c r="J495" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K495" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Farmington Hills</t>
         </is>
       </c>
       <c r="L495" s="3" t="inlineStr">
         <is>
-          <t>29355 Northwestern Hwy #210, Southfield, Michigan, 48034</t>
+          <t>31390 Northwestern Hwy., Ste C, Farmington Hills, Michigan, 48334</t>
         </is>
       </c>
       <c r="M495" s="3" t="n"/>
@@ -33845,7 +33845,7 @@
       </c>
       <c r="D496" s="3" t="inlineStr">
         <is>
-          <t>📝 Jian Zu MD</t>
+          <t>📝 Corewell Internal Medicine Southfield</t>
         </is>
       </c>
       <c r="E496" s="3" t="inlineStr">
@@ -33860,7 +33860,7 @@
       </c>
       <c r="G496" s="2" t="inlineStr">
         <is>
-          <t>85043f4d-a0d7-448b-9a3d-e0943de69dd8</t>
+          <t>5eb6a409-5e7b-430f-a462-af3a919cfc22</t>
         </is>
       </c>
       <c r="H496" s="2" t="inlineStr">
@@ -33883,7 +33883,7 @@
       </c>
       <c r="L496" s="3" t="inlineStr">
         <is>
-          <t>29355 Northwestern Hwy, Southfield, Michigan, 48034</t>
+          <t>29355 Northwestern Hwy #210, Southfield, Michigan, 48034</t>
         </is>
       </c>
       <c r="M496" s="3" t="n"/>
@@ -33905,7 +33905,7 @@
       </c>
       <c r="D497" s="3" t="inlineStr">
         <is>
-          <t>📝 Carson Center Specialty</t>
+          <t>📝 Jian Zu MD</t>
         </is>
       </c>
       <c r="E497" s="3" t="inlineStr">
@@ -33920,7 +33920,7 @@
       </c>
       <c r="G497" s="2" t="inlineStr">
         <is>
-          <t>fe708f7e-ac39-4cb4-91fb-ef244909b360</t>
+          <t>85043f4d-a0d7-448b-9a3d-e0943de69dd8</t>
         </is>
       </c>
       <c r="H497" s="2" t="inlineStr">
@@ -33934,7 +33934,7 @@
         </is>
       </c>
       <c r="J497" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K497" s="2" t="inlineStr">
         <is>
@@ -33943,7 +33943,7 @@
       </c>
       <c r="L497" s="3" t="inlineStr">
         <is>
-          <t>29355 NORTHWESTERN HWY STE 120, SOUTHFIELD, MI, 48034</t>
+          <t>29355 Northwestern Hwy, Southfield, Michigan, 48034</t>
         </is>
       </c>
       <c r="M497" s="3" t="n"/>
@@ -33965,12 +33965,12 @@
       </c>
       <c r="D498" s="3" t="inlineStr">
         <is>
-          <t>📝 ROSE MEDICINE</t>
+          <t>📝 Carson Center Specialty</t>
         </is>
       </c>
       <c r="E498" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 10</t>
+          <t>Tier 1 producer · last check-in Sep 29</t>
         </is>
       </c>
       <c r="F498" s="2" t="inlineStr">
@@ -33980,7 +33980,7 @@
       </c>
       <c r="G498" s="2" t="inlineStr">
         <is>
-          <t>9c2f2817-fae0-4fb0-b943-376aef6fc719</t>
+          <t>fe708f7e-ac39-4cb4-91fb-ef244909b360</t>
         </is>
       </c>
       <c r="H498" s="2" t="inlineStr">
@@ -33994,16 +33994,16 @@
         </is>
       </c>
       <c r="J498" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K498" s="2" t="inlineStr">
         <is>
-          <t>Bingham Farms</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L498" s="3" t="inlineStr">
         <is>
-          <t>31500 TELEGRAPH RD STE 115, BINGHAM FARMS, MI, 48025</t>
+          <t>29355 NORTHWESTERN HWY STE 120, SOUTHFIELD, MI, 48034</t>
         </is>
       </c>
       <c r="M498" s="3" t="n"/>
@@ -34205,45 +34205,45 @@
       </c>
       <c r="D502" s="3" t="inlineStr">
         <is>
-          <t>📝 Corewell URGENT CARE BY WELLSTREET</t>
+          <t>📝 IHA UNION LAKE PEDIATRICS</t>
         </is>
       </c>
       <c r="E502" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Jul 29</t>
+          <t>Tier 1 producer · last check-in Sep 15</t>
         </is>
       </c>
       <c r="F502" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G502" s="2" t="inlineStr">
         <is>
-          <t>5f3e3632-715d-4e1c-b4ca-4c6bc3dac21e</t>
+          <t>905d0bbb-d935-4258-8a1e-2e30d0a25987</t>
         </is>
       </c>
       <c r="H502" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I502" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not sure</t>
         </is>
       </c>
       <c r="J502" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K502" s="2" t="inlineStr">
         <is>
-          <t>Bloomfield Township</t>
+          <t>Commerce Township</t>
         </is>
       </c>
       <c r="L502" s="3" t="inlineStr">
         <is>
-          <t>6543 TELEGRAPH RD, BLOOMFIELD TOWNSHIP, Michigan</t>
+          <t>2630 UNION LAKE RD STE 100, COMMERCE TOWNSHIP, Michigan</t>
         </is>
       </c>
       <c r="M502" s="3" t="n"/>
@@ -34805,12 +34805,12 @@
       </c>
       <c r="D512" s="3" t="inlineStr">
         <is>
-          <t>📝 DMC Orthopedics - Commerce Township</t>
+          <t>White Lake Family Medicine</t>
         </is>
       </c>
       <c r="E512" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 21</t>
+          <t>Tier 1 producer · last check-in Jul 21</t>
         </is>
       </c>
       <c r="F512" s="2" t="inlineStr">
@@ -34820,30 +34820,30 @@
       </c>
       <c r="G512" s="2" t="inlineStr">
         <is>
-          <t>568c9052-985c-48fa-b5bc-44baafba3dea</t>
+          <t>6f873c6d-498d-4d61-b717-d6648675da4e</t>
         </is>
       </c>
       <c r="H512" s="2" t="inlineStr">
         <is>
-          <t>Orthopedic</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I512" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J512" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K512" s="2" t="inlineStr">
         <is>
-          <t>Commerce Township</t>
+          <t>White Lake</t>
         </is>
       </c>
       <c r="L512" s="3" t="inlineStr">
         <is>
-          <t>1 William Carls Drive, Michigan, 48382</t>
+          <t>9178 Highland Rd, White Lake, MI 483864619</t>
         </is>
       </c>
       <c r="M512" s="3" t="n"/>
@@ -34865,12 +34865,12 @@
       </c>
       <c r="D513" s="3" t="inlineStr">
         <is>
-          <t>📝 Providence Park Pediatrics - Novi</t>
+          <t>ALAN L FELDMAN, DO, PC</t>
         </is>
       </c>
       <c r="E513" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 25</t>
+          <t>Tier 1 producer · last check-in May 26</t>
         </is>
       </c>
       <c r="F513" s="2" t="inlineStr">
@@ -34880,17 +34880,17 @@
       </c>
       <c r="G513" s="2" t="inlineStr">
         <is>
-          <t>9db7de95-514d-45c7-8a73-449a08d1d590</t>
+          <t>5d0e63d7-bdd3-445e-a627-ef0ea5dc48f7</t>
         </is>
       </c>
       <c r="H513" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I513" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J513" s="2" t="n">
@@ -34898,12 +34898,12 @@
       </c>
       <c r="K513" s="2" t="inlineStr">
         <is>
-          <t>Novi</t>
+          <t>Commerce Township</t>
         </is>
       </c>
       <c r="L513" s="3" t="inlineStr">
         <is>
-          <t>26850 PROVIDENCE PKWY STE 455, NOVI, Michigan</t>
+          <t>1965 Union Lake Rd, Commerce Township, MI 48382</t>
         </is>
       </c>
       <c r="M513" s="3" t="n"/>
@@ -34925,12 +34925,12 @@
       </c>
       <c r="D514" s="3" t="inlineStr">
         <is>
-          <t>📝 PILLAY INTERNAL MEDICINE ASSOCIATES, PLLC</t>
+          <t>📝 CoreMed - Commerce</t>
         </is>
       </c>
       <c r="E514" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 15</t>
+          <t>Tier 1 producer · last check-in Aug 21</t>
         </is>
       </c>
       <c r="F514" s="2" t="inlineStr">
@@ -34940,7 +34940,7 @@
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>f5f4f354-94f3-42a1-a3be-10f8a64cdaae</t>
+          <t>eab7d954-a523-466a-a75b-3eca7bf9c6d0</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
@@ -34958,12 +34958,12 @@
       </c>
       <c r="K514" s="2" t="inlineStr">
         <is>
-          <t>Walled Lake</t>
+          <t>Commerce Township</t>
         </is>
       </c>
       <c r="L514" s="3" t="inlineStr">
         <is>
-          <t>100 N POND DR STE C, WALLED LAKE, MI, 48390</t>
+          <t>2600 Union Lake Rd suite 140 Commerce Township, Michigan, 48382</t>
         </is>
       </c>
       <c r="M514" s="3" t="n"/>
@@ -34985,12 +34985,12 @@
       </c>
       <c r="D515" s="3" t="inlineStr">
         <is>
-          <t>LAKES INTERNAL MEDICINE - 2150</t>
+          <t>📝 Rodnick Chiropractic</t>
         </is>
       </c>
       <c r="E515" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 10</t>
+          <t>Tier 1 producer · last check-in Sep 15</t>
         </is>
       </c>
       <c r="F515" s="2" t="inlineStr">
@@ -35000,17 +35000,17 @@
       </c>
       <c r="G515" s="2" t="inlineStr">
         <is>
-          <t>8b9ada78-08d8-45f0-8d09-c043db61a6fd</t>
+          <t>97e1431f-4c5b-4ec4-b3a5-47267613937b</t>
         </is>
       </c>
       <c r="H515" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="I515" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J515" s="2" t="n">
@@ -35018,12 +35018,12 @@
       </c>
       <c r="K515" s="2" t="inlineStr">
         <is>
-          <t>West Bloomfield</t>
+          <t>Commerce Charter Township</t>
         </is>
       </c>
       <c r="L515" s="3" t="inlineStr">
         <is>
-          <t>2300 Haggerty Rd Ste 2150, West Bloomfield, MI 48323</t>
+          <t>2685 Union Lake Rd Commerce Charter Twp, Commerce Charter Township, Michigan, 48382</t>
         </is>
       </c>
       <c r="M515" s="3" t="n"/>
@@ -35105,12 +35105,12 @@
       </c>
       <c r="D517" s="3" t="inlineStr">
         <is>
-          <t>📝 Rodnick Chiropractic</t>
+          <t>📝 DMC Orthopedics - Commerce Township</t>
         </is>
       </c>
       <c r="E517" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 15</t>
+          <t>Tier 1 producer · last check-in Aug 21</t>
         </is>
       </c>
       <c r="F517" s="2" t="inlineStr">
@@ -35120,12 +35120,12 @@
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>97e1431f-4c5b-4ec4-b3a5-47267613937b</t>
+          <t>568c9052-985c-48fa-b5bc-44baafba3dea</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Orthopedic</t>
         </is>
       </c>
       <c r="I517" s="2" t="inlineStr">
@@ -35134,16 +35134,16 @@
         </is>
       </c>
       <c r="J517" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K517" s="2" t="inlineStr">
         <is>
-          <t>Commerce Charter Township</t>
+          <t>Commerce Township</t>
         </is>
       </c>
       <c r="L517" s="3" t="inlineStr">
         <is>
-          <t>2685 Union Lake Rd Commerce Charter Twp, Commerce Charter Township, Michigan, 48382</t>
+          <t>1 William Carls Drive, Michigan, 48382</t>
         </is>
       </c>
       <c r="M517" s="3" t="n"/>
@@ -35165,12 +35165,12 @@
       </c>
       <c r="D518" s="3" t="inlineStr">
         <is>
-          <t>📝 IHA UNION LAKE PEDIATRICS</t>
+          <t>📝 Providence Park Pediatrics - Novi</t>
         </is>
       </c>
       <c r="E518" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 15</t>
+          <t>Tier 1 producer · last check-in Sep 25</t>
         </is>
       </c>
       <c r="F518" s="2" t="inlineStr">
@@ -35180,7 +35180,7 @@
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>905d0bbb-d935-4258-8a1e-2e30d0a25987</t>
+          <t>9db7de95-514d-45c7-8a73-449a08d1d590</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
@@ -35190,7 +35190,7 @@
       </c>
       <c r="I518" s="2" t="inlineStr">
         <is>
-          <t>Not sure</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J518" s="2" t="n">
@@ -35198,12 +35198,12 @@
       </c>
       <c r="K518" s="2" t="inlineStr">
         <is>
-          <t>Commerce Township</t>
+          <t>Novi</t>
         </is>
       </c>
       <c r="L518" s="3" t="inlineStr">
         <is>
-          <t>2630 UNION LAKE RD STE 100, COMMERCE TOWNSHIP, Michigan</t>
+          <t>26850 PROVIDENCE PKWY STE 455, NOVI, Michigan</t>
         </is>
       </c>
       <c r="M518" s="3" t="n"/>
@@ -35225,12 +35225,12 @@
       </c>
       <c r="D519" s="3" t="inlineStr">
         <is>
-          <t>📝 CoreMed - Commerce</t>
+          <t>📝 PILLAY INTERNAL MEDICINE ASSOCIATES, PLLC</t>
         </is>
       </c>
       <c r="E519" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 21</t>
+          <t>Tier 1 producer · last check-in Sep 15</t>
         </is>
       </c>
       <c r="F519" s="2" t="inlineStr">
@@ -35240,7 +35240,7 @@
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>eab7d954-a523-466a-a75b-3eca7bf9c6d0</t>
+          <t>f5f4f354-94f3-42a1-a3be-10f8a64cdaae</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
@@ -35258,12 +35258,12 @@
       </c>
       <c r="K519" s="2" t="inlineStr">
         <is>
-          <t>Commerce Township</t>
+          <t>Walled Lake</t>
         </is>
       </c>
       <c r="L519" s="3" t="inlineStr">
         <is>
-          <t>2600 Union Lake Rd suite 140 Commerce Township, Michigan, 48382</t>
+          <t>100 N POND DR STE C, WALLED LAKE, MI, 48390</t>
         </is>
       </c>
       <c r="M519" s="3" t="n"/>
@@ -35285,12 +35285,12 @@
       </c>
       <c r="D520" s="3" t="inlineStr">
         <is>
-          <t>ALAN L FELDMAN, DO, PC</t>
+          <t>LAKES INTERNAL MEDICINE - 2150</t>
         </is>
       </c>
       <c r="E520" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in May 26</t>
+          <t>Tier 1 producer · last check-in Sep 10</t>
         </is>
       </c>
       <c r="F520" s="2" t="inlineStr">
@@ -35300,7 +35300,7 @@
       </c>
       <c r="G520" s="2" t="inlineStr">
         <is>
-          <t>5d0e63d7-bdd3-445e-a627-ef0ea5dc48f7</t>
+          <t>8b9ada78-08d8-45f0-8d09-c043db61a6fd</t>
         </is>
       </c>
       <c r="H520" s="2" t="inlineStr">
@@ -35318,12 +35318,12 @@
       </c>
       <c r="K520" s="2" t="inlineStr">
         <is>
-          <t>Commerce Township</t>
+          <t>West Bloomfield</t>
         </is>
       </c>
       <c r="L520" s="3" t="inlineStr">
         <is>
-          <t>1965 Union Lake Rd, Commerce Township, MI 48382</t>
+          <t>2300 Haggerty Rd Ste 2150, West Bloomfield, MI 48323</t>
         </is>
       </c>
       <c r="M520" s="3" t="n"/>
@@ -35345,45 +35345,45 @@
       </c>
       <c r="D521" s="3" t="inlineStr">
         <is>
-          <t>📝 HEALING HANDS URGENT CARE</t>
+          <t>MICHIGAN PREMIER INTERNISTS</t>
         </is>
       </c>
       <c r="E521" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Jul 30</t>
+          <t>Tier 1 producer · last check-in Oct 5</t>
         </is>
       </c>
       <c r="F521" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G521" s="2" t="inlineStr">
         <is>
-          <t>ed1959ed-68b4-4788-bfa4-24c1e6d994d6</t>
+          <t>1a1e59ec-5621-4caa-a9e9-b4d86b5218e7</t>
         </is>
       </c>
       <c r="H521" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I521" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J521" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K521" s="2" t="inlineStr">
         <is>
-          <t>Sylvan Lake</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L521" s="3" t="inlineStr">
         <is>
-          <t>2157 ORCHARD LAKE RD, SYLVAN LAKE, Michigan</t>
+          <t>29877 Telegraph Rd Ste 200, Southfield, MI 48034</t>
         </is>
       </c>
       <c r="M521" s="3" t="n"/>
@@ -35405,12 +35405,12 @@
       </c>
       <c r="D522" s="3" t="inlineStr">
         <is>
-          <t>Oakland Medical Center</t>
+          <t>Franklin Medical Consultants</t>
         </is>
       </c>
       <c r="E522" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 1</t>
+          <t>Tier 1 producer · last check-in Oct 5</t>
         </is>
       </c>
       <c r="F522" s="2" t="inlineStr">
@@ -35420,7 +35420,7 @@
       </c>
       <c r="G522" s="2" t="inlineStr">
         <is>
-          <t>77bba5d4-d050-4705-b292-6e3a8a78dec8</t>
+          <t>559bee40-1fa3-437d-9e4b-692838015293</t>
         </is>
       </c>
       <c r="H522" s="2" t="inlineStr">
@@ -35438,12 +35438,12 @@
       </c>
       <c r="K522" s="2" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L522" s="3" t="inlineStr">
         <is>
-          <t>115 E Long Lake Rd, Troy, MI 48085</t>
+          <t>29829 Telegraph Road, Southfield, MI 48034</t>
         </is>
       </c>
       <c r="M522" s="3" t="n"/>
@@ -35465,12 +35465,12 @@
       </c>
       <c r="D523" s="3" t="inlineStr">
         <is>
-          <t>📝 Kashat Urgent care</t>
+          <t>📝 DEIGHTON FAMILY PRACTICE - use this one</t>
         </is>
       </c>
       <c r="E523" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 8</t>
+          <t>Tier 1 producer · last check-in Sep 29</t>
         </is>
       </c>
       <c r="F523" s="2" t="inlineStr">
@@ -35480,12 +35480,12 @@
       </c>
       <c r="G523" s="2" t="inlineStr">
         <is>
-          <t>0b9485b1-39bd-4f21-8222-387834af8472</t>
+          <t>a6779fd4-289a-49f7-8602-76dc1bf5764c</t>
         </is>
       </c>
       <c r="H523" s="2" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I523" s="2" t="inlineStr">
@@ -35498,12 +35498,12 @@
       </c>
       <c r="K523" s="2" t="inlineStr">
         <is>
-          <t>Sterling Heights</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L523" s="3" t="inlineStr">
         <is>
-          <t>35200 Dequindre Road, Sterling Heights, Michigan, 48310</t>
+          <t>22250 PROVIDENCE DR STE 500, SOUTHFIELD, Michigan</t>
         </is>
       </c>
       <c r="M523" s="3" t="n"/>
@@ -35585,7 +35585,7 @@
       </c>
       <c r="D525" s="3" t="inlineStr">
         <is>
-          <t>ASCENSION MACOMB OAKLAND HOSPITAL MOTOR CITY INTERNISTS</t>
+          <t>📝 Kashat Urgent care</t>
         </is>
       </c>
       <c r="E525" s="3" t="inlineStr">
@@ -35600,17 +35600,17 @@
       </c>
       <c r="G525" s="2" t="inlineStr">
         <is>
-          <t>dc78e75f-e0d1-4c67-8de9-8ea4f13f15a1</t>
+          <t>0b9485b1-39bd-4f21-8222-387834af8472</t>
         </is>
       </c>
       <c r="H525" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="I525" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J525" s="2" t="n">
@@ -35618,12 +35618,12 @@
       </c>
       <c r="K525" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="L525" s="3" t="inlineStr">
         <is>
-          <t>11885 E 12 Mile Rd Ste 200B, Warren, MI 48093</t>
+          <t>35200 Dequindre Road, Sterling Heights, Michigan, 48310</t>
         </is>
       </c>
       <c r="M525" s="3" t="n"/>
@@ -35645,7 +35645,7 @@
       </c>
       <c r="D526" s="3" t="inlineStr">
         <is>
-          <t>📝 Michigan Compassionate Care</t>
+          <t>ASCENSION MACOMB OAKLAND HOSPITAL MOTOR CITY INTERNISTS</t>
         </is>
       </c>
       <c r="E526" s="3" t="inlineStr">
@@ -35660,21 +35660,21 @@
       </c>
       <c r="G526" s="2" t="inlineStr">
         <is>
-          <t>33d0c0aa-7d47-450d-9673-71acb651321c</t>
+          <t>dc78e75f-e0d1-4c67-8de9-8ea4f13f15a1</t>
         </is>
       </c>
       <c r="H526" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I526" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J526" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K526" s="2" t="inlineStr">
         <is>
@@ -35683,7 +35683,7 @@
       </c>
       <c r="L526" s="3" t="inlineStr">
         <is>
-          <t>28401 Hoover, Warren, Michigan, 48093</t>
+          <t>11885 E 12 Mile Rd Ste 200B, Warren, MI 48093</t>
         </is>
       </c>
       <c r="M526" s="3" t="n"/>
@@ -35705,7 +35705,7 @@
       </c>
       <c r="D527" s="3" t="inlineStr">
         <is>
-          <t>📝 FERRIS, MARY C, MEDICAL GROUP</t>
+          <t>📝 Michigan Compassionate Care</t>
         </is>
       </c>
       <c r="E527" s="3" t="inlineStr">
@@ -35720,7 +35720,7 @@
       </c>
       <c r="G527" s="2" t="inlineStr">
         <is>
-          <t>a5a045ce-889d-4018-81f5-3fd8d3d7af6b</t>
+          <t>33d0c0aa-7d47-450d-9673-71acb651321c</t>
         </is>
       </c>
       <c r="H527" s="2" t="inlineStr">
@@ -35734,7 +35734,7 @@
         </is>
       </c>
       <c r="J527" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K527" s="2" t="inlineStr">
         <is>
@@ -35743,7 +35743,7 @@
       </c>
       <c r="L527" s="3" t="inlineStr">
         <is>
-          <t>28111 HOOVER RD STE 1A, WARREN, Michigan</t>
+          <t>28401 Hoover, Warren, Michigan, 48093</t>
         </is>
       </c>
       <c r="M527" s="3" t="n"/>
@@ -35765,7 +35765,7 @@
       </c>
       <c r="D528" s="3" t="inlineStr">
         <is>
-          <t>Hoover Primary Care Medical Group</t>
+          <t>📝 FERRIS, MARY C, MEDICAL GROUP</t>
         </is>
       </c>
       <c r="E528" s="3" t="inlineStr">
@@ -35780,17 +35780,17 @@
       </c>
       <c r="G528" s="2" t="inlineStr">
         <is>
-          <t>d2472b07-69ea-403b-b954-d5d8227b1364</t>
+          <t>a5a045ce-889d-4018-81f5-3fd8d3d7af6b</t>
         </is>
       </c>
       <c r="H528" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I528" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J528" s="2" t="n">
@@ -35803,7 +35803,7 @@
       </c>
       <c r="L528" s="3" t="inlineStr">
         <is>
-          <t>28111 Hoover Rd, Ste 5A Warren, Mi 48093, Usa, Warren, MI 48093</t>
+          <t>28111 HOOVER RD STE 1A, WARREN, Michigan</t>
         </is>
       </c>
       <c r="M528" s="3" t="n"/>
@@ -35825,7 +35825,7 @@
       </c>
       <c r="D529" s="3" t="inlineStr">
         <is>
-          <t>Macomb Neurology Associates</t>
+          <t>Hoover Primary Care Medical Group</t>
         </is>
       </c>
       <c r="E529" s="3" t="inlineStr">
@@ -35840,12 +35840,12 @@
       </c>
       <c r="G529" s="2" t="inlineStr">
         <is>
-          <t>1023090552</t>
+          <t>d2472b07-69ea-403b-b954-d5d8227b1364</t>
         </is>
       </c>
       <c r="H529" s="2" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I529" s="2" t="inlineStr">
@@ -35863,7 +35863,7 @@
       </c>
       <c r="L529" s="3" t="inlineStr">
         <is>
-          <t>27427 Schoenherr Rd, Warren, MI 48088</t>
+          <t>28111 Hoover Rd, Ste 5A Warren, Mi 48093, Usa, Warren, MI 48093</t>
         </is>
       </c>
       <c r="M529" s="3" t="n"/>
@@ -35885,27 +35885,27 @@
       </c>
       <c r="D530" s="3" t="inlineStr">
         <is>
-          <t>Emcura Immediate Care - Grosse Pointe</t>
+          <t>Macomb Neurology Associates</t>
         </is>
       </c>
       <c r="E530" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Jun 3</t>
+          <t>Tier 1 producer · last check-in Oct 8</t>
         </is>
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G530" s="2" t="inlineStr">
         <is>
-          <t>bf549ea4-0d9c-4877-927c-ed3f99bf0988</t>
+          <t>1023090552</t>
         </is>
       </c>
       <c r="H530" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="I530" s="2" t="inlineStr">
@@ -35914,16 +35914,16 @@
         </is>
       </c>
       <c r="J530" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K530" s="2" t="inlineStr">
         <is>
-          <t>Grosse Pointe Woods</t>
+          <t>Warren</t>
         </is>
       </c>
       <c r="L530" s="3" t="inlineStr">
         <is>
-          <t>20599 Mack Ave, Grosse Pointe Woods, MI 48236</t>
+          <t>27427 Schoenherr Rd, Warren, MI 48088</t>
         </is>
       </c>
       <c r="M530" s="3" t="n"/>
@@ -35945,12 +35945,12 @@
       </c>
       <c r="D531" s="3" t="inlineStr">
         <is>
-          <t>📝 DEIGHTON FAMILY PRACTICE - use this one</t>
+          <t>📝 Pulmonary &amp; Medical Associates</t>
         </is>
       </c>
       <c r="E531" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 29</t>
+          <t>Tier 1 producer · last check-in Oct 8</t>
         </is>
       </c>
       <c r="F531" s="2" t="inlineStr">
@@ -35960,7 +35960,7 @@
       </c>
       <c r="G531" s="2" t="inlineStr">
         <is>
-          <t>a6779fd4-289a-49f7-8602-76dc1bf5764c</t>
+          <t>dda630a5-9d61-49cd-bec6-61084e47ddb9</t>
         </is>
       </c>
       <c r="H531" s="2" t="inlineStr">
@@ -35974,16 +35974,16 @@
         </is>
       </c>
       <c r="J531" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K531" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Warren</t>
         </is>
       </c>
       <c r="L531" s="3" t="inlineStr">
         <is>
-          <t>22250 PROVIDENCE DR STE 500, SOUTHFIELD, Michigan</t>
+          <t>27472 Schoenherr Rd #100, Warren, MI, 48088</t>
         </is>
       </c>
       <c r="M531" s="3" t="n"/>
@@ -36365,7 +36365,7 @@
       </c>
       <c r="D538" s="3" t="inlineStr">
         <is>
-          <t>📝 Pulmonary &amp; Medical Associates</t>
+          <t>📝 Northpointe Pediatrics</t>
         </is>
       </c>
       <c r="E538" s="3" t="inlineStr">
@@ -36380,12 +36380,12 @@
       </c>
       <c r="G538" s="2" t="inlineStr">
         <is>
-          <t>dda630a5-9d61-49cd-bec6-61084e47ddb9</t>
+          <t>31b0544c-cc2c-4479-9df9-b11748ecefc7</t>
         </is>
       </c>
       <c r="H538" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I538" s="2" t="inlineStr">
@@ -36394,7 +36394,7 @@
         </is>
       </c>
       <c r="J538" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K538" s="2" t="inlineStr">
         <is>
@@ -36403,7 +36403,7 @@
       </c>
       <c r="L538" s="3" t="inlineStr">
         <is>
-          <t>27472 Schoenherr Rd #100, Warren, MI, 48088</t>
+          <t>30061 Schoenherr Rd, Warren, Michigan, 48088</t>
         </is>
       </c>
       <c r="M538" s="3" t="n"/>
@@ -36725,12 +36725,12 @@
       </c>
       <c r="D544" s="3" t="inlineStr">
         <is>
-          <t>📝 Center For Hollistic Medicine</t>
+          <t>Burhani Medical Center - use this one</t>
         </is>
       </c>
       <c r="E544" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 10</t>
+          <t>Tier 1 producer · last check-in May 13</t>
         </is>
       </c>
       <c r="F544" s="2" t="inlineStr">
@@ -36740,17 +36740,17 @@
       </c>
       <c r="G544" s="2" t="inlineStr">
         <is>
-          <t>42b038b0-949b-46be-8843-e02868bb894a</t>
+          <t>3ade325e-79e3-41bc-a8b9-565bcfc77f2c</t>
         </is>
       </c>
       <c r="H544" s="2" t="inlineStr">
         <is>
-          <t>Other / Verify</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I544" s="2" t="inlineStr">
         <is>
-          <t>Not sure</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J544" s="2" t="n">
@@ -36758,12 +36758,12 @@
       </c>
       <c r="K544" s="2" t="inlineStr">
         <is>
-          <t>West Bloomfield</t>
+          <t>Farmington Hills</t>
         </is>
       </c>
       <c r="L544" s="3" t="inlineStr">
         <is>
-          <t>6089 W MAPLE RD STE 200, WEST BLOOMFIELD, Michigan</t>
+          <t>32910 West 13 Mile Road, A101, Farmington Hills, MI 48334</t>
         </is>
       </c>
       <c r="M544" s="3" t="n"/>
@@ -36785,12 +36785,12 @@
       </c>
       <c r="D545" s="3" t="inlineStr">
         <is>
-          <t>Burhani Medical Center - use this one</t>
+          <t>📝 Henry Ford Primary Care - Orchard Lake Road North</t>
         </is>
       </c>
       <c r="E545" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in May 13</t>
+          <t>Tier 1 producer · last check-in Aug 13</t>
         </is>
       </c>
       <c r="F545" s="2" t="inlineStr">
@@ -36800,21 +36800,21 @@
       </c>
       <c r="G545" s="2" t="inlineStr">
         <is>
-          <t>3ade325e-79e3-41bc-a8b9-565bcfc77f2c</t>
+          <t>960ab807-be26-45c0-bbf9-135ef0a45ae0</t>
         </is>
       </c>
       <c r="H545" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I545" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J545" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K545" s="2" t="inlineStr">
         <is>
@@ -36823,7 +36823,7 @@
       </c>
       <c r="L545" s="3" t="inlineStr">
         <is>
-          <t>32910 West 13 Mile Road, A101, Farmington Hills, MI 48334</t>
+          <t>27970 ORCHARD LAKE RD, FARMINGTON HILLS, Michigan, 48334</t>
         </is>
       </c>
       <c r="M545" s="3" t="n"/>
@@ -36845,12 +36845,12 @@
       </c>
       <c r="D546" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Primary Care - Orchard Lake Road North</t>
+          <t>📝 FARMINGTON HILLS  FAMILY PHYSICIANS, PLLC</t>
         </is>
       </c>
       <c r="E546" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 13</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F546" s="2" t="inlineStr">
@@ -36860,7 +36860,7 @@
       </c>
       <c r="G546" s="2" t="inlineStr">
         <is>
-          <t>960ab807-be26-45c0-bbf9-135ef0a45ae0</t>
+          <t>cc6d8767-1fad-4a5b-b658-38a67ea47a1c</t>
         </is>
       </c>
       <c r="H546" s="2" t="inlineStr">
@@ -36874,7 +36874,7 @@
         </is>
       </c>
       <c r="J546" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K546" s="2" t="inlineStr">
         <is>
@@ -36883,7 +36883,7 @@
       </c>
       <c r="L546" s="3" t="inlineStr">
         <is>
-          <t>27970 ORCHARD LAKE RD, FARMINGTON HILLS, Michigan, 48334</t>
+          <t>29930 W 12 MILE RD STE 6, FARMINGTON HILLS, Michigan</t>
         </is>
       </c>
       <c r="M546" s="3" t="n"/>
@@ -36905,12 +36905,12 @@
       </c>
       <c r="D547" s="3" t="inlineStr">
         <is>
-          <t>📝 FARMINGTON HILLS  FAMILY PHYSICIANS, PLLC</t>
+          <t>📝 Legend Health - Now One Health</t>
         </is>
       </c>
       <c r="E547" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 19</t>
+          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 29</t>
         </is>
       </c>
       <c r="F547" s="2" t="inlineStr">
@@ -36920,7 +36920,7 @@
       </c>
       <c r="G547" s="2" t="inlineStr">
         <is>
-          <t>cc6d8767-1fad-4a5b-b658-38a67ea47a1c</t>
+          <t>078d2fa6-e81c-41d1-95f2-04234d511192</t>
         </is>
       </c>
       <c r="H547" s="2" t="inlineStr">
@@ -36934,16 +36934,16 @@
         </is>
       </c>
       <c r="J547" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K547" s="2" t="inlineStr">
         <is>
-          <t>Farmington Hills</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L547" s="3" t="inlineStr">
         <is>
-          <t>29930 W 12 MILE RD STE 6, FARMINGTON HILLS, Michigan</t>
+          <t>29201 Telegraph Rd, ste 403, Southfield, MI, 48034</t>
         </is>
       </c>
       <c r="M547" s="3" t="n"/>
@@ -36965,12 +36965,12 @@
       </c>
       <c r="D548" s="3" t="inlineStr">
         <is>
-          <t>📝 Legend Health - Now One Health</t>
+          <t>📝 ORCHARD PRIMARY CARE</t>
         </is>
       </c>
       <c r="E548" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 29</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F548" s="2" t="inlineStr">
@@ -36980,7 +36980,7 @@
       </c>
       <c r="G548" s="2" t="inlineStr">
         <is>
-          <t>078d2fa6-e81c-41d1-95f2-04234d511192</t>
+          <t>ba00dba0-20f9-440b-8df0-799ade91a785</t>
         </is>
       </c>
       <c r="H548" s="2" t="inlineStr">
@@ -36998,12 +36998,12 @@
       </c>
       <c r="K548" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Farmington Hills</t>
         </is>
       </c>
       <c r="L548" s="3" t="inlineStr">
         <is>
-          <t>29201 Telegraph Rd, ste 403, Southfield, MI, 48034</t>
+          <t>30852 W 10 MILE RD, FARMINGTON HILLS, MI, 48336</t>
         </is>
       </c>
       <c r="M548" s="3" t="n"/>
@@ -37805,45 +37805,45 @@
       </c>
       <c r="D562" s="3" t="inlineStr">
         <is>
-          <t>MALI AND MALI PEDIATRICS - use this one</t>
+          <t>📝 1st Choice Urgent Care</t>
         </is>
       </c>
       <c r="E562" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 1</t>
+          <t>Prospect · last check-in Aug 25</t>
         </is>
       </c>
       <c r="F562" s="2" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G562" s="2" t="inlineStr">
         <is>
-          <t>2e26f7de-9e76-464a-a322-fbef639b64d7</t>
+          <t>e7cc65bc-b486-4ee3-9c39-431666859cbd</t>
         </is>
       </c>
       <c r="H562" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="I562" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J562" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K562" s="2" t="inlineStr">
         <is>
-          <t>Sterling Heights</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L562" s="3" t="inlineStr">
         <is>
-          <t>44344 Dequindre Rd Ste 510, Sterling Heights, MI nan</t>
+          <t>29628 Southfield Road, Southfield, Michigan, 48076</t>
         </is>
       </c>
       <c r="M562" s="3" t="n"/>
@@ -37865,12 +37865,12 @@
       </c>
       <c r="D563" s="3" t="inlineStr">
         <is>
-          <t>📝 Michigan Primary Care - Sterling Heights</t>
+          <t>📝 Lifetime Family Care</t>
         </is>
       </c>
       <c r="E563" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 8</t>
+          <t>Tier 1 producer · last check-in Aug 26</t>
         </is>
       </c>
       <c r="F563" s="2" t="inlineStr">
@@ -37880,7 +37880,7 @@
       </c>
       <c r="G563" s="2" t="inlineStr">
         <is>
-          <t>ce3b56cf-1381-41d0-b067-752448464958</t>
+          <t>b70053c3-f0fd-41de-9386-95fcc448a738</t>
         </is>
       </c>
       <c r="H563" s="2" t="inlineStr">
@@ -37894,16 +37894,16 @@
         </is>
       </c>
       <c r="J563" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K563" s="2" t="inlineStr">
         <is>
-          <t>Sterling Heights</t>
+          <t>Madison Heights</t>
         </is>
       </c>
       <c r="L563" s="3" t="inlineStr">
         <is>
-          <t>41400 Dequindre Rd, ste 121, Sterling Heights, Michigan, 48314</t>
+          <t>26393 Dequindre Rd, Madison Heights, Michigan, 48071</t>
         </is>
       </c>
       <c r="M563" s="3" t="n"/>
@@ -37925,12 +37925,12 @@
       </c>
       <c r="D564" s="3" t="inlineStr">
         <is>
-          <t>Concentra Urgent Care - Sterling Heights</t>
+          <t>📝 Get Well Urgent Care Madison Heights</t>
         </is>
       </c>
       <c r="E564" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 7</t>
+          <t>Tier 1 producer · last check-in Aug 25</t>
         </is>
       </c>
       <c r="F564" s="2" t="inlineStr">
@@ -37940,30 +37940,30 @@
       </c>
       <c r="G564" s="2" t="inlineStr">
         <is>
-          <t>dc6067ed-60f7-4ae5-8b5b-7b8b03095484</t>
+          <t>346a1335-a97f-4a1a-9847-77f9e71383c3</t>
         </is>
       </c>
       <c r="H564" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="I564" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J564" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K564" s="2" t="inlineStr">
         <is>
-          <t>Sterling Heights</t>
+          <t>Madison Heights</t>
         </is>
       </c>
       <c r="L564" s="3" t="inlineStr">
         <is>
-          <t>39333 Van Dyke Ave, Sterling Heights, Mi 48313, United States, Sterling Heights, MI 48313</t>
+          <t>350 E 12 Mile Rd, Madison Heights, Michigan, 48071</t>
         </is>
       </c>
       <c r="M564" s="3" t="n"/>
@@ -37985,12 +37985,12 @@
       </c>
       <c r="D565" s="3" t="inlineStr">
         <is>
-          <t>📝 Get Well Urgent Care - Sterling Heights</t>
+          <t>📝 Sterling Physicians</t>
         </is>
       </c>
       <c r="E565" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 3</t>
+          <t>Tier 1 producer · last check-in Oct 8</t>
         </is>
       </c>
       <c r="F565" s="2" t="inlineStr">
@@ -38000,12 +38000,12 @@
       </c>
       <c r="G565" s="2" t="inlineStr">
         <is>
-          <t>1bcc2e23-5fc1-428c-ad41-dc35c5345bf7</t>
+          <t>1972593499</t>
         </is>
       </c>
       <c r="H565" s="2" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I565" s="2" t="inlineStr">
@@ -38023,7 +38023,7 @@
       </c>
       <c r="L565" s="3" t="inlineStr">
         <is>
-          <t>2567 Metro Parkway, Sterling Heights, Michigan, 48310</t>
+          <t>36040 Dequindre Road, Sterling Heights, Michigan, 48310</t>
         </is>
       </c>
       <c r="M565" s="3" t="n"/>
@@ -38045,7 +38045,7 @@
       </c>
       <c r="D566" s="3" t="inlineStr">
         <is>
-          <t>📝 Tri-County Medical Clinic</t>
+          <t>📝 Get Well Urgent Care - Sterling Heights</t>
         </is>
       </c>
       <c r="E566" s="3" t="inlineStr">
@@ -38060,12 +38060,12 @@
       </c>
       <c r="G566" s="2" t="inlineStr">
         <is>
-          <t>1386634749</t>
+          <t>1bcc2e23-5fc1-428c-ad41-dc35c5345bf7</t>
         </is>
       </c>
       <c r="H566" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent Care</t>
         </is>
       </c>
       <c r="I566" s="2" t="inlineStr">
@@ -38083,7 +38083,7 @@
       </c>
       <c r="L566" s="3" t="inlineStr">
         <is>
-          <t>37450 DeQuindre Rd, Sterling Heights, MI, 48310</t>
+          <t>2567 Metro Parkway, Sterling Heights, Michigan, 48310</t>
         </is>
       </c>
       <c r="M566" s="3" t="n"/>
@@ -38165,12 +38165,12 @@
       </c>
       <c r="D568" s="3" t="inlineStr">
         <is>
-          <t>📝 Sterling Physicians</t>
+          <t>📝 Tri-County Medical Clinic</t>
         </is>
       </c>
       <c r="E568" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 8</t>
+          <t>Tier 1 producer · last check-in Sep 3</t>
         </is>
       </c>
       <c r="F568" s="2" t="inlineStr">
@@ -38180,7 +38180,7 @@
       </c>
       <c r="G568" s="2" t="inlineStr">
         <is>
-          <t>1972593499</t>
+          <t>1386634749</t>
         </is>
       </c>
       <c r="H568" s="2" t="inlineStr">
@@ -38203,7 +38203,7 @@
       </c>
       <c r="L568" s="3" t="inlineStr">
         <is>
-          <t>36040 Dequindre Road, Sterling Heights, Michigan, 48310</t>
+          <t>37450 DeQuindre Rd, Sterling Heights, MI, 48310</t>
         </is>
       </c>
       <c r="M568" s="3" t="n"/>
@@ -38225,12 +38225,12 @@
       </c>
       <c r="D569" s="3" t="inlineStr">
         <is>
-          <t>📝 Get Well Urgent Care Madison Heights</t>
+          <t>📝 Michigan Primary Care - Sterling Heights</t>
         </is>
       </c>
       <c r="E569" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 25</t>
+          <t>Tier 1 producer · last check-in Oct 8</t>
         </is>
       </c>
       <c r="F569" s="2" t="inlineStr">
@@ -38240,12 +38240,12 @@
       </c>
       <c r="G569" s="2" t="inlineStr">
         <is>
-          <t>346a1335-a97f-4a1a-9847-77f9e71383c3</t>
+          <t>ce3b56cf-1381-41d0-b067-752448464958</t>
         </is>
       </c>
       <c r="H569" s="2" t="inlineStr">
         <is>
-          <t>Urgent Care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I569" s="2" t="inlineStr">
@@ -38254,16 +38254,16 @@
         </is>
       </c>
       <c r="J569" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K569" s="2" t="inlineStr">
         <is>
-          <t>Madison Heights</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="L569" s="3" t="inlineStr">
         <is>
-          <t>350 E 12 Mile Rd, Madison Heights, Michigan, 48071</t>
+          <t>41400 Dequindre Rd, ste 121, Sterling Heights, Michigan, 48314</t>
         </is>
       </c>
       <c r="M569" s="3" t="n"/>
@@ -38285,45 +38285,45 @@
       </c>
       <c r="D570" s="3" t="inlineStr">
         <is>
-          <t>📝 Corewell Health Urgent Care - Warren West</t>
+          <t>MALI AND MALI PEDIATRICS - use this one</t>
         </is>
       </c>
       <c r="E570" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Aug 26</t>
+          <t>Tier 1 producer · last check-in Oct 1</t>
         </is>
       </c>
       <c r="F570" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G570" s="2" t="inlineStr">
         <is>
-          <t>9152636b-052e-44f2-ab21-a7abf86561ff</t>
+          <t>2e26f7de-9e76-464a-a322-fbef639b64d7</t>
         </is>
       </c>
       <c r="H570" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I570" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J570" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K570" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="L570" s="3" t="inlineStr">
         <is>
-          <t>28324 Dequindre Road, Warren, Michigan, 48092</t>
+          <t>44344 Dequindre Rd Ste 510, Sterling Heights, MI nan</t>
         </is>
       </c>
       <c r="M570" s="3" t="n"/>
@@ -38345,12 +38345,12 @@
       </c>
       <c r="D571" s="3" t="inlineStr">
         <is>
-          <t>📝 Lifetime Family Care</t>
+          <t>Concentra Urgent Care - Sterling Heights</t>
         </is>
       </c>
       <c r="E571" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 26</t>
+          <t>Tier 1 producer · last check-in Oct 7</t>
         </is>
       </c>
       <c r="F571" s="2" t="inlineStr">
@@ -38360,30 +38360,30 @@
       </c>
       <c r="G571" s="2" t="inlineStr">
         <is>
-          <t>b70053c3-f0fd-41de-9386-95fcc448a738</t>
+          <t>dc6067ed-60f7-4ae5-8b5b-7b8b03095484</t>
         </is>
       </c>
       <c r="H571" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="I571" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J571" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K571" s="2" t="inlineStr">
         <is>
-          <t>Madison Heights</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="L571" s="3" t="inlineStr">
         <is>
-          <t>26393 Dequindre Rd, Madison Heights, Michigan, 48071</t>
+          <t>39333 Van Dyke Ave, Sterling Heights, Mi 48313, United States, Sterling Heights, MI 48313</t>
         </is>
       </c>
       <c r="M571" s="3" t="n"/>
@@ -38585,12 +38585,12 @@
       </c>
       <c r="D575" s="3" t="inlineStr">
         <is>
-          <t>📝 Powers Family Medicine</t>
+          <t>📝 Brentwood Pediatric Associates</t>
         </is>
       </c>
       <c r="E575" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 19</t>
+          <t>Tier 1 producer · last check-in Sep 11</t>
         </is>
       </c>
       <c r="F575" s="2" t="inlineStr">
@@ -38600,12 +38600,12 @@
       </c>
       <c r="G575" s="2" t="inlineStr">
         <is>
-          <t>00-761-7874</t>
+          <t>9dfbaa38-07b2-4017-9d71-ff4cd2ce42f7</t>
         </is>
       </c>
       <c r="H575" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I575" s="2" t="inlineStr">
@@ -38614,16 +38614,16 @@
         </is>
       </c>
       <c r="J575" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K575" s="2" t="inlineStr">
         <is>
-          <t>Farmington Hills</t>
+          <t>Livonia</t>
         </is>
       </c>
       <c r="L575" s="3" t="inlineStr">
         <is>
-          <t>23700 Orchard Lake Rd, Farmington Hills, MI, 48336-2559</t>
+          <t>33215 W Seven Mile Rd, Livonia, Michigan, 48152</t>
         </is>
       </c>
       <c r="M575" s="3" t="n"/>
@@ -38645,12 +38645,12 @@
       </c>
       <c r="D576" s="3" t="inlineStr">
         <is>
-          <t>📝 ORCHARD PRIMARY CARE</t>
+          <t>📝 Triumph chiropractic</t>
         </is>
       </c>
       <c r="E576" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 19</t>
+          <t>Tier 1 producer · last check-in Sep 16</t>
         </is>
       </c>
       <c r="F576" s="2" t="inlineStr">
@@ -38660,12 +38660,12 @@
       </c>
       <c r="G576" s="2" t="inlineStr">
         <is>
-          <t>ba00dba0-20f9-440b-8df0-799ade91a785</t>
+          <t>d99edd32-fb45-4528-94d3-645792efefa1</t>
         </is>
       </c>
       <c r="H576" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Other / Verify</t>
         </is>
       </c>
       <c r="I576" s="2" t="inlineStr">
@@ -38674,16 +38674,16 @@
         </is>
       </c>
       <c r="J576" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K576" s="2" t="inlineStr">
         <is>
-          <t>Farmington Hills</t>
+          <t>Livonia</t>
         </is>
       </c>
       <c r="L576" s="3" t="inlineStr">
         <is>
-          <t>30852 W 10 MILE RD, FARMINGTON HILLS, MI, 48336</t>
+          <t>20216 Farmington Road, Livonia, Michigan, 48152</t>
         </is>
       </c>
       <c r="M576" s="3" t="n"/>
@@ -38705,27 +38705,27 @@
       </c>
       <c r="D577" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Go Health Urgent Care</t>
+          <t>📝 Powers Family Medicine</t>
         </is>
       </c>
       <c r="E577" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in May 27</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F577" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G577" s="2" t="inlineStr">
         <is>
-          <t>14f29ff1-cd7e-4e90-b5c7-b1114551c5b9</t>
+          <t>00-761-7874</t>
         </is>
       </c>
       <c r="H577" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I577" s="2" t="inlineStr">
@@ -38734,16 +38734,16 @@
         </is>
       </c>
       <c r="J577" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K577" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Farmington Hills</t>
         </is>
       </c>
       <c r="L577" s="3" t="inlineStr">
         <is>
-          <t>28670 Telegraph Road, Southfield, Michigan, 48034</t>
+          <t>23700 Orchard Lake Rd, Farmington Hills, MI, 48336-2559</t>
         </is>
       </c>
       <c r="M577" s="3" t="n"/>
@@ -38765,36 +38765,36 @@
       </c>
       <c r="D578" s="3" t="inlineStr">
         <is>
-          <t>Franklin Medical Consultants</t>
+          <t>📝 Henry Ford Go Health Urgent Care</t>
         </is>
       </c>
       <c r="E578" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 5</t>
+          <t>Prospect · last check-in May 27</t>
         </is>
       </c>
       <c r="F578" s="2" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G578" s="2" t="inlineStr">
         <is>
-          <t>559bee40-1fa3-437d-9e4b-692838015293</t>
+          <t>14f29ff1-cd7e-4e90-b5c7-b1114551c5b9</t>
         </is>
       </c>
       <c r="H578" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="I578" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J578" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K578" s="2" t="inlineStr">
         <is>
@@ -38803,7 +38803,7 @@
       </c>
       <c r="L578" s="3" t="inlineStr">
         <is>
-          <t>29829 Telegraph Road, Southfield, MI 48034</t>
+          <t>28670 Telegraph Road, Southfield, Michigan, 48034</t>
         </is>
       </c>
       <c r="M578" s="3" t="n"/>
@@ -38825,12 +38825,12 @@
       </c>
       <c r="D579" s="3" t="inlineStr">
         <is>
-          <t>MICHIGAN PREMIER INTERNISTS</t>
+          <t>📝 ROSE MEDICINE</t>
         </is>
       </c>
       <c r="E579" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 5</t>
+          <t>Tier 1 producer · last check-in Sep 10</t>
         </is>
       </c>
       <c r="F579" s="2" t="inlineStr">
@@ -38840,30 +38840,30 @@
       </c>
       <c r="G579" s="2" t="inlineStr">
         <is>
-          <t>1a1e59ec-5621-4caa-a9e9-b4d86b5218e7</t>
+          <t>9c2f2817-fae0-4fb0-b943-376aef6fc719</t>
         </is>
       </c>
       <c r="H579" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I579" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J579" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K579" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Bingham Farms</t>
         </is>
       </c>
       <c r="L579" s="3" t="inlineStr">
         <is>
-          <t>29877 Telegraph Rd Ste 200, Southfield, MI 48034</t>
+          <t>31500 TELEGRAPH RD STE 115, BINGHAM FARMS, MI, 48025</t>
         </is>
       </c>
       <c r="M579" s="3" t="n"/>
@@ -39005,7 +39005,7 @@
       </c>
       <c r="D582" s="3" t="inlineStr">
         <is>
-          <t>White Lake Family Medicine</t>
+          <t>Core Med  - White Lake</t>
         </is>
       </c>
       <c r="E582" s="3" t="inlineStr">
@@ -39020,7 +39020,7 @@
       </c>
       <c r="G582" s="2" t="inlineStr">
         <is>
-          <t>6f873c6d-498d-4d61-b717-d6648675da4e</t>
+          <t>ecbe00dd-1c49-4028-a575-d8852e23deba</t>
         </is>
       </c>
       <c r="H582" s="2" t="inlineStr">
@@ -39034,16 +39034,16 @@
         </is>
       </c>
       <c r="J582" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K582" s="2" t="inlineStr">
         <is>
-          <t>White Lake</t>
+          <t>White Lake Charter Township</t>
         </is>
       </c>
       <c r="L582" s="3" t="inlineStr">
         <is>
-          <t>9178 Highland Rd, White Lake, MI 483864619</t>
+          <t>8355 Highland Road, White Lake Charter Township, MI 48386</t>
         </is>
       </c>
       <c r="M582" s="3" t="n"/>
@@ -39185,7 +39185,7 @@
       </c>
       <c r="D585" s="3" t="inlineStr">
         <is>
-          <t>📝 Corewell Internal Medicine Southfield</t>
+          <t>📝 Carson Center Specialty</t>
         </is>
       </c>
       <c r="E585" s="3" t="inlineStr">
@@ -39200,7 +39200,7 @@
       </c>
       <c r="G585" s="2" t="inlineStr">
         <is>
-          <t>5eb6a409-5e7b-430f-a462-af3a919cfc22</t>
+          <t>fe708f7e-ac39-4cb4-91fb-ef244909b360</t>
         </is>
       </c>
       <c r="H585" s="2" t="inlineStr">
@@ -39214,7 +39214,7 @@
         </is>
       </c>
       <c r="J585" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K585" s="2" t="inlineStr">
         <is>
@@ -39223,7 +39223,7 @@
       </c>
       <c r="L585" s="3" t="inlineStr">
         <is>
-          <t>29355 Northwestern Hwy #210, Southfield, Michigan, 48034</t>
+          <t>29355 NORTHWESTERN HWY STE 120, SOUTHFIELD, MI, 48034</t>
         </is>
       </c>
       <c r="M585" s="3" t="n"/>
@@ -39245,12 +39245,12 @@
       </c>
       <c r="D586" s="3" t="inlineStr">
         <is>
-          <t>📝 Triumph chiropractic</t>
+          <t>📝 Jian Zu MD</t>
         </is>
       </c>
       <c r="E586" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 16</t>
+          <t>Tier 1 producer · last check-in Sep 29</t>
         </is>
       </c>
       <c r="F586" s="2" t="inlineStr">
@@ -39260,12 +39260,12 @@
       </c>
       <c r="G586" s="2" t="inlineStr">
         <is>
-          <t>d99edd32-fb45-4528-94d3-645792efefa1</t>
+          <t>85043f4d-a0d7-448b-9a3d-e0943de69dd8</t>
         </is>
       </c>
       <c r="H586" s="2" t="inlineStr">
         <is>
-          <t>Other / Verify</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I586" s="2" t="inlineStr">
@@ -39274,16 +39274,16 @@
         </is>
       </c>
       <c r="J586" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Livonia</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L586" s="3" t="inlineStr">
         <is>
-          <t>20216 Farmington Road, Livonia, Michigan, 48152</t>
+          <t>29355 Northwestern Hwy, Southfield, Michigan, 48034</t>
         </is>
       </c>
       <c r="M586" s="3" t="n"/>
@@ -39305,12 +39305,12 @@
       </c>
       <c r="D587" s="3" t="inlineStr">
         <is>
-          <t>📝 Brentwood Pediatric Associates</t>
+          <t>📝 Corewell Internal Medicine Southfield</t>
         </is>
       </c>
       <c r="E587" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 11</t>
+          <t>Tier 1 producer · last check-in Sep 29</t>
         </is>
       </c>
       <c r="F587" s="2" t="inlineStr">
@@ -39320,12 +39320,12 @@
       </c>
       <c r="G587" s="2" t="inlineStr">
         <is>
-          <t>9dfbaa38-07b2-4017-9d71-ff4cd2ce42f7</t>
+          <t>5eb6a409-5e7b-430f-a462-af3a919cfc22</t>
         </is>
       </c>
       <c r="H587" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I587" s="2" t="inlineStr">
@@ -39338,12 +39338,12 @@
       </c>
       <c r="K587" s="2" t="inlineStr">
         <is>
-          <t>Livonia</t>
+          <t>Southfield</t>
         </is>
       </c>
       <c r="L587" s="3" t="inlineStr">
         <is>
-          <t>33215 W Seven Mile Rd, Livonia, Michigan, 48152</t>
+          <t>29355 Northwestern Hwy #210, Southfield, Michigan, 48034</t>
         </is>
       </c>
       <c r="M587" s="3" t="n"/>
@@ -39365,7 +39365,7 @@
       </c>
       <c r="D588" s="3" t="inlineStr">
         <is>
-          <t>📝 AGHA INTERNAL MEDICINE AND ASSOCIATES, PC</t>
+          <t>📝 Beaumont Medical Center - Redford</t>
         </is>
       </c>
       <c r="E588" s="3" t="inlineStr">
@@ -39380,7 +39380,7 @@
       </c>
       <c r="G588" s="2" t="inlineStr">
         <is>
-          <t>85fd21cb-8cbc-4ead-9b3d-0cdbecdf7638</t>
+          <t>03095e36-e586-4709-8cd8-440a98b9bcd7</t>
         </is>
       </c>
       <c r="H588" s="2" t="inlineStr">
@@ -39394,16 +39394,16 @@
         </is>
       </c>
       <c r="J588" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Livonia</t>
+          <t>Redford Charter Township</t>
         </is>
       </c>
       <c r="L588" s="3" t="inlineStr">
         <is>
-          <t>15604 FARMINGTON RD, LIVONIA, MI, 48154</t>
+          <t>15540 Beech Daly, Redford Charter Township, Michigan, 48239</t>
         </is>
       </c>
       <c r="M588" s="3" t="n"/>
@@ -39425,7 +39425,7 @@
       </c>
       <c r="D589" s="3" t="inlineStr">
         <is>
-          <t>📝 Beaumont Medical Center - Redford</t>
+          <t>📝 ARBOR LANE FAMILY PHYSICIANS</t>
         </is>
       </c>
       <c r="E589" s="3" t="inlineStr">
@@ -39440,7 +39440,7 @@
       </c>
       <c r="G589" s="2" t="inlineStr">
         <is>
-          <t>03095e36-e586-4709-8cd8-440a98b9bcd7</t>
+          <t>ff61f8fa-5169-42e7-aafe-f189027c5f3a</t>
         </is>
       </c>
       <c r="H589" s="2" t="inlineStr">
@@ -39454,16 +39454,16 @@
         </is>
       </c>
       <c r="J589" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K589" s="2" t="inlineStr">
         <is>
-          <t>Redford Charter Township</t>
+          <t>Redford</t>
         </is>
       </c>
       <c r="L589" s="3" t="inlineStr">
         <is>
-          <t>15540 Beech Daly, Redford Charter Township, Michigan, 48239</t>
+          <t>24224 JOY RD STE 100, REDFORD, Michigan</t>
         </is>
       </c>
       <c r="M589" s="3" t="n"/>
@@ -39485,7 +39485,7 @@
       </c>
       <c r="D590" s="3" t="inlineStr">
         <is>
-          <t>📝 ARBOR LANE FAMILY PHYSICIANS</t>
+          <t>📝 AGHA INTERNAL MEDICINE AND ASSOCIATES, PC</t>
         </is>
       </c>
       <c r="E590" s="3" t="inlineStr">
@@ -39500,7 +39500,7 @@
       </c>
       <c r="G590" s="2" t="inlineStr">
         <is>
-          <t>ff61f8fa-5169-42e7-aafe-f189027c5f3a</t>
+          <t>85fd21cb-8cbc-4ead-9b3d-0cdbecdf7638</t>
         </is>
       </c>
       <c r="H590" s="2" t="inlineStr">
@@ -39518,12 +39518,12 @@
       </c>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Redford</t>
+          <t>Livonia</t>
         </is>
       </c>
       <c r="L590" s="3" t="inlineStr">
         <is>
-          <t>24224 JOY RD STE 100, REDFORD, Michigan</t>
+          <t>15604 FARMINGTON RD, LIVONIA, MI, 48154</t>
         </is>
       </c>
       <c r="M590" s="3" t="n"/>
@@ -42005,45 +42005,45 @@
       </c>
       <c r="D632" s="3" t="inlineStr">
         <is>
-          <t>📝 Universal Clinic &amp; Urgent Care</t>
+          <t>Clinton Preferred Pediatrics</t>
         </is>
       </c>
       <c r="E632" s="3" t="inlineStr">
         <is>
-          <t>Prospect · last check-in Sep 2</t>
+          <t>Tier 1 producer · last check-in Oct 7</t>
         </is>
       </c>
       <c r="F632" s="2" t="inlineStr">
         <is>
-          <t>Prospect</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="G632" s="2" t="inlineStr">
         <is>
-          <t>d689dac9-8b56-4f6e-9ba4-8bf3eb8e3550</t>
+          <t>abd1a370-f826-48dd-a800-9a15983f52e8</t>
         </is>
       </c>
       <c r="H632" s="2" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="I632" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J632" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K632" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L632" s="3" t="inlineStr">
         <is>
-          <t>4600 14 Mile Rd ste 1, Warren, Michigan, 48092</t>
+          <t>15500 19 Mile Rd Suite 300, Clinton Township, MI 48038</t>
         </is>
       </c>
       <c r="M632" s="3" t="n"/>
@@ -42065,12 +42065,12 @@
       </c>
       <c r="D633" s="3" t="inlineStr">
         <is>
-          <t>📝 Henry Ford Warren Family Physicians</t>
+          <t>📝 Macomb Internal Medicine</t>
         </is>
       </c>
       <c r="E633" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 26</t>
+          <t>Tier 1 producer · last check-in Jul 10</t>
         </is>
       </c>
       <c r="F633" s="2" t="inlineStr">
@@ -42080,7 +42080,7 @@
       </c>
       <c r="G633" s="2" t="inlineStr">
         <is>
-          <t>6771a475-3022-40fd-9db9-b8e0291f7082</t>
+          <t>5271bbd8-dfe5-4d54-a0a2-f5547050cafe</t>
         </is>
       </c>
       <c r="H633" s="2" t="inlineStr">
@@ -42094,16 +42094,16 @@
         </is>
       </c>
       <c r="J633" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K633" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L633" s="3" t="inlineStr">
         <is>
-          <t>11270 East Thirteen Mile Road, Warren, Michigan, 48093</t>
+          <t>15520 19 Mile Road, Suite 480, Clinton Township, MI, 48038</t>
         </is>
       </c>
       <c r="M633" s="3" t="n"/>
@@ -42125,12 +42125,12 @@
       </c>
       <c r="D634" s="3" t="inlineStr">
         <is>
-          <t>📝 DIAB AND KINNER INTERNAL MEDICINE, PC- use</t>
+          <t>📝 Swetech Medical Center</t>
         </is>
       </c>
       <c r="E634" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 27</t>
+          <t>Tier 1 producer · last check-in Oct 7</t>
         </is>
       </c>
       <c r="F634" s="2" t="inlineStr">
@@ -42140,7 +42140,7 @@
       </c>
       <c r="G634" s="2" t="inlineStr">
         <is>
-          <t>954353cc-a941-4b77-90f3-f3fb1c62e161</t>
+          <t>1255427209</t>
         </is>
       </c>
       <c r="H634" s="2" t="inlineStr">
@@ -42158,12 +42158,12 @@
       </c>
       <c r="K634" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L634" s="3" t="inlineStr">
         <is>
-          <t>29703 HOOVER RD STE A, WARREN, Michigan, 48093</t>
+          <t>43600 Garfield Rd, Clinton Township, Michigan, 48038</t>
         </is>
       </c>
       <c r="M634" s="3" t="n"/>
@@ -42185,12 +42185,12 @@
       </c>
       <c r="D635" s="3" t="inlineStr">
         <is>
-          <t>📝 Northpointe Pediatrics</t>
+          <t>Macomb Pediatrics - Clinton Township</t>
         </is>
       </c>
       <c r="E635" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 8</t>
+          <t>Tier 1 producer · last check-in Oct 7</t>
         </is>
       </c>
       <c r="F635" s="2" t="inlineStr">
@@ -42200,7 +42200,7 @@
       </c>
       <c r="G635" s="2" t="inlineStr">
         <is>
-          <t>31b0544c-cc2c-4479-9df9-b11748ecefc7</t>
+          <t>9e284312-a8af-43ff-9b39-5d4a8c1ed834</t>
         </is>
       </c>
       <c r="H635" s="2" t="inlineStr">
@@ -42210,7 +42210,7 @@
       </c>
       <c r="I635" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J635" s="2" t="n">
@@ -42218,12 +42218,12 @@
       </c>
       <c r="K635" s="2" t="inlineStr">
         <is>
-          <t>Warren</t>
+          <t>Clinton Township</t>
         </is>
       </c>
       <c r="L635" s="3" t="inlineStr">
         <is>
-          <t>30061 Schoenherr Rd, Warren, Michigan, 48088</t>
+          <t>39200 Garfield Rd Suite E Clinton Twp, Clinton Township, MI 48038</t>
         </is>
       </c>
       <c r="M635" s="3" t="n"/>
@@ -42305,12 +42305,12 @@
       </c>
       <c r="D637" s="3" t="inlineStr">
         <is>
-          <t>Macomb Pediatrics - Clinton Township</t>
+          <t>📝 Legacy Family Medicine</t>
         </is>
       </c>
       <c r="E637" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 7</t>
+          <t>Tier 1 producer · tier Tier 2→Tier 1 (Sep 22) · last check-in Sep 8</t>
         </is>
       </c>
       <c r="F637" s="2" t="inlineStr">
@@ -42320,17 +42320,17 @@
       </c>
       <c r="G637" s="2" t="inlineStr">
         <is>
-          <t>9e284312-a8af-43ff-9b39-5d4a8c1ed834</t>
+          <t>1558340356</t>
         </is>
       </c>
       <c r="H637" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I637" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J637" s="2" t="n">
@@ -42338,12 +42338,12 @@
       </c>
       <c r="K637" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Sterling Heights</t>
         </is>
       </c>
       <c r="L637" s="3" t="inlineStr">
         <is>
-          <t>39200 Garfield Rd Suite E Clinton Twp, Clinton Township, MI 48038</t>
+          <t>35429 Schoenherr Rd, Sterling Heights, MI, 48312</t>
         </is>
       </c>
       <c r="M637" s="3" t="n"/>
@@ -42365,12 +42365,12 @@
       </c>
       <c r="D638" s="3" t="inlineStr">
         <is>
-          <t>📝 Macomb Internal Medicine</t>
+          <t>📝 Henry Ford Warren Family Physicians</t>
         </is>
       </c>
       <c r="E638" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Jul 10</t>
+          <t>Tier 1 producer · last check-in Aug 26</t>
         </is>
       </c>
       <c r="F638" s="2" t="inlineStr">
@@ -42380,7 +42380,7 @@
       </c>
       <c r="G638" s="2" t="inlineStr">
         <is>
-          <t>5271bbd8-dfe5-4d54-a0a2-f5547050cafe</t>
+          <t>6771a475-3022-40fd-9db9-b8e0291f7082</t>
         </is>
       </c>
       <c r="H638" s="2" t="inlineStr">
@@ -42394,16 +42394,16 @@
         </is>
       </c>
       <c r="J638" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K638" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Warren</t>
         </is>
       </c>
       <c r="L638" s="3" t="inlineStr">
         <is>
-          <t>15520 19 Mile Road, Suite 480, Clinton Township, MI, 48038</t>
+          <t>11270 East Thirteen Mile Road, Warren, Michigan, 48093</t>
         </is>
       </c>
       <c r="M638" s="3" t="n"/>
@@ -42425,12 +42425,12 @@
       </c>
       <c r="D639" s="3" t="inlineStr">
         <is>
-          <t>Clinton Preferred Pediatrics</t>
+          <t>📝 DIAB AND KINNER INTERNAL MEDICINE, PC- use</t>
         </is>
       </c>
       <c r="E639" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 7</t>
+          <t>Tier 1 producer · last check-in Aug 27</t>
         </is>
       </c>
       <c r="F639" s="2" t="inlineStr">
@@ -42440,17 +42440,17 @@
       </c>
       <c r="G639" s="2" t="inlineStr">
         <is>
-          <t>abd1a370-f826-48dd-a800-9a15983f52e8</t>
+          <t>954353cc-a941-4b77-90f3-f3fb1c62e161</t>
         </is>
       </c>
       <c r="H639" s="2" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="I639" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J639" s="2" t="n">
@@ -42458,12 +42458,12 @@
       </c>
       <c r="K639" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Warren</t>
         </is>
       </c>
       <c r="L639" s="3" t="inlineStr">
         <is>
-          <t>15500 19 Mile Rd Suite 300, Clinton Township, MI 48038</t>
+          <t>29703 HOOVER RD STE A, WARREN, Michigan, 48093</t>
         </is>
       </c>
       <c r="M639" s="3" t="n"/>
@@ -42485,45 +42485,45 @@
       </c>
       <c r="D640" s="3" t="inlineStr">
         <is>
-          <t>📝 Swetech Medical Center</t>
+          <t>Emcura Immediate Care - Grosse Pointe</t>
         </is>
       </c>
       <c r="E640" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Oct 7</t>
+          <t>Prospect · last check-in Jun 3</t>
         </is>
       </c>
       <c r="F640" s="2" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G640" s="2" t="inlineStr">
         <is>
-          <t>1255427209</t>
+          <t>bf549ea4-0d9c-4877-927c-ed3f99bf0988</t>
         </is>
       </c>
       <c r="H640" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="I640" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J640" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K640" s="2" t="inlineStr">
         <is>
-          <t>Clinton Township</t>
+          <t>Grosse Pointe Woods</t>
         </is>
       </c>
       <c r="L640" s="3" t="inlineStr">
         <is>
-          <t>43600 Garfield Rd, Clinton Township, Michigan, 48038</t>
+          <t>20599 Mack Ave, Grosse Pointe Woods, MI 48236</t>
         </is>
       </c>
       <c r="M640" s="3" t="n"/>
@@ -43145,12 +43145,12 @@
       </c>
       <c r="D651" s="3" t="inlineStr">
         <is>
-          <t>Core Med  - White Lake</t>
+          <t>📝 Center For Hollistic Medicine</t>
         </is>
       </c>
       <c r="E651" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Jul 21</t>
+          <t>Tier 1 producer · last check-in Sep 10</t>
         </is>
       </c>
       <c r="F651" s="2" t="inlineStr">
@@ -43160,17 +43160,17 @@
       </c>
       <c r="G651" s="2" t="inlineStr">
         <is>
-          <t>ecbe00dd-1c49-4028-a575-d8852e23deba</t>
+          <t>42b038b0-949b-46be-8843-e02868bb894a</t>
         </is>
       </c>
       <c r="H651" s="2" t="inlineStr">
         <is>
-          <t>PCP / IM / FM</t>
+          <t>Other / Verify</t>
         </is>
       </c>
       <c r="I651" s="2" t="inlineStr">
         <is>
-          <t>Added Sep 3 (Joe — referral receipts)</t>
+          <t>Not sure</t>
         </is>
       </c>
       <c r="J651" s="2" t="n">
@@ -43178,12 +43178,12 @@
       </c>
       <c r="K651" s="2" t="inlineStr">
         <is>
-          <t>White Lake Charter Township</t>
+          <t>West Bloomfield</t>
         </is>
       </c>
       <c r="L651" s="3" t="inlineStr">
         <is>
-          <t>8355 Highland Road, White Lake Charter Township, MI 48386</t>
+          <t>6089 W MAPLE RD STE 200, WEST BLOOMFIELD, Michigan</t>
         </is>
       </c>
       <c r="M651" s="3" t="n"/>
@@ -43265,27 +43265,27 @@
       </c>
       <c r="D653" s="3" t="inlineStr">
         <is>
-          <t>📝 Legacy Family Care</t>
+          <t>📝 Corewell URGENT CARE BY WELLSTREET</t>
         </is>
       </c>
       <c r="E653" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 19</t>
+          <t>Prospect · last check-in Jul 29</t>
         </is>
       </c>
       <c r="F653" s="2" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Prospect</t>
         </is>
       </c>
       <c r="G653" s="2" t="inlineStr">
         <is>
-          <t>6a6a4408-2a28-4e5b-aea6-b70d4b47d57c</t>
+          <t>5f3e3632-715d-4e1c-b4ca-4c6bc3dac21e</t>
         </is>
       </c>
       <c r="H653" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="I653" s="2" t="inlineStr">
@@ -43294,16 +43294,16 @@
         </is>
       </c>
       <c r="J653" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K653" s="2" t="inlineStr">
         <is>
-          <t>Farmington Hills</t>
+          <t>Bloomfield Township</t>
         </is>
       </c>
       <c r="L653" s="3" t="inlineStr">
         <is>
-          <t>23800 Orchard Lake Rd suite 202, Farmington Hills, Michigan, 48336</t>
+          <t>6543 TELEGRAPH RD, BLOOMFIELD TOWNSHIP, Michigan</t>
         </is>
       </c>
       <c r="M653" s="3" t="n"/>
@@ -43325,12 +43325,12 @@
       </c>
       <c r="D654" s="3" t="inlineStr">
         <is>
-          <t>📝 Jian Zu MD</t>
+          <t>📝 TWIN LAKES MEDICAL ASSOCIATES, PC</t>
         </is>
       </c>
       <c r="E654" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 29</t>
+          <t>Tier 1 producer · last check-in Sep 16</t>
         </is>
       </c>
       <c r="F654" s="2" t="inlineStr">
@@ -43340,7 +43340,7 @@
       </c>
       <c r="G654" s="2" t="inlineStr">
         <is>
-          <t>85043f4d-a0d7-448b-9a3d-e0943de69dd8</t>
+          <t>e7b52c83-5403-4607-98fb-61ffa473ccc4</t>
         </is>
       </c>
       <c r="H654" s="2" t="inlineStr">
@@ -43358,12 +43358,12 @@
       </c>
       <c r="K654" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Bloomfield</t>
         </is>
       </c>
       <c r="L654" s="3" t="inlineStr">
         <is>
-          <t>29355 Northwestern Hwy, Southfield, Michigan, 48034</t>
+          <t>43700 WOODWARD AVE STE 206, BLOOMFIELD, Michigan, MI 48302</t>
         </is>
       </c>
       <c r="M654" s="3" t="n"/>
@@ -43385,12 +43385,12 @@
       </c>
       <c r="D655" s="3" t="inlineStr">
         <is>
-          <t>📝 Carson Center Specialty</t>
+          <t>Oakland Medical Center</t>
         </is>
       </c>
       <c r="E655" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 29</t>
+          <t>Tier 1 producer · last check-in Oct 1</t>
         </is>
       </c>
       <c r="F655" s="2" t="inlineStr">
@@ -43400,30 +43400,30 @@
       </c>
       <c r="G655" s="2" t="inlineStr">
         <is>
-          <t>fe708f7e-ac39-4cb4-91fb-ef244909b360</t>
+          <t>77bba5d4-d050-4705-b292-6e3a8a78dec8</t>
         </is>
       </c>
       <c r="H655" s="2" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>PCP / IM / FM</t>
         </is>
       </c>
       <c r="I655" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Added Sep 3 (Joe — referral receipts)</t>
         </is>
       </c>
       <c r="J655" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K655" s="2" t="inlineStr">
         <is>
-          <t>Southfield</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="L655" s="3" t="inlineStr">
         <is>
-          <t>29355 NORTHWESTERN HWY STE 120, SOUTHFIELD, MI, 48034</t>
+          <t>115 E Long Lake Rd, Troy, MI 48085</t>
         </is>
       </c>
       <c r="M655" s="3" t="n"/>
@@ -43445,12 +43445,12 @@
       </c>
       <c r="D656" s="3" t="inlineStr">
         <is>
-          <t>📝 ROSE MEDICINE</t>
+          <t>📝 Brigid Healthcare</t>
         </is>
       </c>
       <c r="E656" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 10</t>
+          <t>Tier 1 producer · last check-in Sep 14</t>
         </is>
       </c>
       <c r="F656" s="2" t="inlineStr">
@@ -43460,7 +43460,7 @@
       </c>
       <c r="G656" s="2" t="inlineStr">
         <is>
-          <t>9c2f2817-fae0-4fb0-b943-376aef6fc719</t>
+          <t>63bf16ad-3645-45fb-8f1d-e1eb3a131efc</t>
         </is>
       </c>
       <c r="H656" s="2" t="inlineStr">
@@ -43474,16 +43474,16 @@
         </is>
       </c>
       <c r="J656" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K656" s="2" t="inlineStr">
         <is>
-          <t>Bingham Farms</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="L656" s="3" t="inlineStr">
         <is>
-          <t>31500 TELEGRAPH RD STE 115, BINGHAM FARMS, MI, 48025</t>
+          <t>3456 Rochester Rd, Troy, Michigan, 48083</t>
         </is>
       </c>
       <c r="M656" s="3" t="n"/>
@@ -43505,12 +43505,12 @@
       </c>
       <c r="D657" s="3" t="inlineStr">
         <is>
-          <t>📝 Berkley Urgent Care</t>
+          <t>📝 MedPro Primary Care</t>
         </is>
       </c>
       <c r="E657" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 10</t>
+          <t>Tier 1 producer · last check-in Aug 26</t>
         </is>
       </c>
       <c r="F657" s="2" t="inlineStr">
@@ -43520,7 +43520,7 @@
       </c>
       <c r="G657" s="2" t="inlineStr">
         <is>
-          <t>1774d7c7-2d8b-42c6-9dac-78c2a9cf3ed8</t>
+          <t>eebb725b-b031-43b9-a3d7-bfa83d77bc18</t>
         </is>
       </c>
       <c r="H657" s="2" t="inlineStr">
@@ -43534,16 +43534,16 @@
         </is>
       </c>
       <c r="J657" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K657" s="2" t="inlineStr">
         <is>
-          <t>Berkley</t>
+          <t>Madison Heights</t>
         </is>
       </c>
       <c r="L657" s="3" t="inlineStr">
         <is>
-          <t>3270 Greenfield Rd, Berkley, Michigan, 48072</t>
+          <t>31005 John R Rd suite a, Madison Heights, Michigan, 48071</t>
         </is>
       </c>
       <c r="M657" s="3" t="n"/>
@@ -43565,12 +43565,12 @@
       </c>
       <c r="D658" s="3" t="inlineStr">
         <is>
-          <t>📝 MedPro Primary Care</t>
+          <t>📝 Berkley Urgent Care</t>
         </is>
       </c>
       <c r="E658" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Aug 26</t>
+          <t>Tier 1 producer · last check-in Sep 10</t>
         </is>
       </c>
       <c r="F658" s="2" t="inlineStr">
@@ -43580,7 +43580,7 @@
       </c>
       <c r="G658" s="2" t="inlineStr">
         <is>
-          <t>eebb725b-b031-43b9-a3d7-bfa83d77bc18</t>
+          <t>1774d7c7-2d8b-42c6-9dac-78c2a9cf3ed8</t>
         </is>
       </c>
       <c r="H658" s="2" t="inlineStr">
@@ -43594,16 +43594,16 @@
         </is>
       </c>
       <c r="J658" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K658" s="2" t="inlineStr">
         <is>
-          <t>Madison Heights</t>
+          <t>Berkley</t>
         </is>
       </c>
       <c r="L658" s="3" t="inlineStr">
         <is>
-          <t>31005 John R Rd suite a, Madison Heights, Michigan, 48071</t>
+          <t>3270 Greenfield Rd, Berkley, Michigan, 48072</t>
         </is>
       </c>
       <c r="M658" s="3" t="n"/>
@@ -43625,12 +43625,12 @@
       </c>
       <c r="D659" s="3" t="inlineStr">
         <is>
-          <t>📝 Brigid Healthcare</t>
+          <t>📝 Legacy Family Care</t>
         </is>
       </c>
       <c r="E659" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 14</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F659" s="2" t="inlineStr">
@@ -43640,7 +43640,7 @@
       </c>
       <c r="G659" s="2" t="inlineStr">
         <is>
-          <t>63bf16ad-3645-45fb-8f1d-e1eb3a131efc</t>
+          <t>6a6a4408-2a28-4e5b-aea6-b70d4b47d57c</t>
         </is>
       </c>
       <c r="H659" s="2" t="inlineStr">
@@ -43654,16 +43654,16 @@
         </is>
       </c>
       <c r="J659" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K659" s="2" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Farmington Hills</t>
         </is>
       </c>
       <c r="L659" s="3" t="inlineStr">
         <is>
-          <t>3456 Rochester Rd, Troy, Michigan, 48083</t>
+          <t>23800 Orchard Lake Rd suite 202, Farmington Hills, Michigan, 48336</t>
         </is>
       </c>
       <c r="M659" s="3" t="n"/>
@@ -43685,12 +43685,12 @@
       </c>
       <c r="D660" s="3" t="inlineStr">
         <is>
-          <t>📝 TWIN LAKES MEDICAL ASSOCIATES, PC</t>
+          <t>📝 Village Medical Farmington</t>
         </is>
       </c>
       <c r="E660" s="3" t="inlineStr">
         <is>
-          <t>Tier 1 producer · last check-in Sep 16</t>
+          <t>Tier 1 producer · last check-in Aug 19</t>
         </is>
       </c>
       <c r="F660" s="2" t="inlineStr">
@@ -43700,7 +43700,7 @@
       </c>
       <c r="G660" s="2" t="inlineStr">
         <is>
-          <t>e7b52c83-5403-4607-98fb-61ffa473ccc4</t>
+          <t>8a6ae159-0242-4272-b933-bd11fc117733</t>
         </is>
       </c>
       <c r="H660" s="2" t="inlineStr">
@@ -43714,16 +43714,16 @@
         </is>
       </c>
       <c r="J660" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K660" s="2" t="inlineStr">
         <is>
-          <t>Bloomfield</t>
+          <t>Farmington</t>
         </is>
       </c>
       <c r="L660" s="3" t="inlineStr">
         <is>
-          <t>43700 WOODWARD AVE STE 206, BLOOMFIELD, Michigan, MI 48302</t>
+          <t>23133 Orchard Lake Rd, Farmington, Michigan, 48336</t>
         </is>
       </c>
       <c r="M660" s="3" t="n"/>
@@ -66345,7 +66345,7 @@
         <v>46</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>14</v>
@@ -66354,7 +66354,7 @@
         <v>3</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -66370,7 +66370,7 @@
         <v>50</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>6</v>
@@ -66379,7 +66379,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -66420,7 +66420,7 @@
         <v>49</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>12</v>
@@ -66429,7 +66429,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>